<commit_message>
fix: docs-reference CI no longer tries to push to protected main
Replace the auto-commit-to-main step with a diff-check that emits a
warning annotation if docs/pattern-reference.xlsx is stale. The file
is now updated locally and included in each PR diff — branch protection
blocks direct github-actions[bot] pushes, so auto-commit can never work.
Also regenerate docs/pattern-reference.xlsx with the latest engine.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/pattern-reference.xlsx
+++ b/docs/pattern-reference.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F77"/>
+  <dimension ref="A1:F90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1530,10 +1530,48 @@
         </is>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" s="1" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B62" s="1" t="inlineStr"/>
+      <c r="C62" s="1" t="inlineStr"/>
+      <c r="D62" s="1" t="inlineStr"/>
+      <c r="E62" s="1" t="inlineStr">
+        <is>
+          <t>── BOUNDED DATA + SKIP_IF (fixed-slot templates) ───────────────────────</t>
+        </is>
+      </c>
+    </row>
     <row r="63">
-      <c r="A63" s="6" t="inlineStr">
-        <is>
-          <t>END:</t>
+      <c r="A63" s="1" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B63" s="1" t="inlineStr"/>
+      <c r="C63" s="1" t="inlineStr"/>
+      <c r="D63" s="1" t="inlineStr"/>
+      <c r="E63" s="1" t="inlineStr">
+        <is>
+          <t>Use DATA:{n,m} when the template pre-allocates a fixed number of rows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="1" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B64" s="1" t="inlineStr"/>
+      <c r="C64" s="1" t="inlineStr"/>
+      <c r="D64" s="1" t="inlineStr"/>
+      <c r="E64" s="1" t="inlineStr">
+        <is>
+          <t>n = min total physical rows expected, m = max total rows to scan.</t>
         </is>
       </c>
     </row>
@@ -1548,7 +1586,7 @@
       <c r="D65" s="1" t="inlineStr"/>
       <c r="E65" s="1" t="inlineStr">
         <is>
-          <t>── QUICK REFERENCE ──────────────────────────────────────────────</t>
+          <t>SKIP_IF: rows matching the condition are silently excluded from output</t>
         </is>
       </c>
     </row>
@@ -1558,211 +1596,378 @@
           <t>doc:</t>
         </is>
       </c>
-      <c r="B66" s="1" t="inlineStr">
+      <c r="B66" s="1" t="inlineStr"/>
+      <c r="C66" s="1" t="inlineStr"/>
+      <c r="D66" s="1" t="inlineStr"/>
+      <c r="E66" s="1" t="inlineStr">
+        <is>
+          <t>but still count toward the {n,m} bounds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="1" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B67" s="1" t="inlineStr"/>
+      <c r="C67" s="1" t="inlineStr"/>
+      <c r="D67" s="1" t="inlineStr"/>
+      <c r="E67" s="1" t="inlineStr">
+        <is>
+          <t>SKIP_IF is only valid with DATA:{n,m}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="7" t="inlineStr">
+        <is>
+          <t>table:1</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="8" t="n"/>
+      <c r="B69" s="8" t="inlineStr">
+        <is>
+          <t>HEADER:1</t>
+        </is>
+      </c>
+      <c r="C69" s="8" t="inlineStr">
+        <is>
+          <t>col_item</t>
+        </is>
+      </c>
+      <c r="D69" s="8" t="inlineStr">
+        <is>
+          <t>col_qty</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="8" t="n"/>
+      <c r="B70" s="8" t="inlineStr">
+        <is>
+          <t>SKIP_IF</t>
+        </is>
+      </c>
+      <c r="C70" s="8" t="inlineStr">
+        <is>
+          <t>EMPTY</t>
+        </is>
+      </c>
+      <c r="D70" s="8" t="inlineStr">
+        <is>
+          <t>IGNORE</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="8" t="n"/>
+      <c r="B71" s="8" t="inlineStr">
+        <is>
+          <t>DATA:{0,15}</t>
+        </is>
+      </c>
+      <c r="C71" s="8" t="inlineStr">
+        <is>
+          <t>line.item</t>
+        </is>
+      </c>
+      <c r="D71" s="8" t="inlineStr">
+        <is>
+          <t>line.qty</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="8" t="n"/>
+      <c r="B72" s="8" t="inlineStr">
+        <is>
+          <t>FOOTER:1</t>
+        </is>
+      </c>
+      <c r="C72" s="8" t="inlineStr">
+        <is>
+          <t>lbl_total</t>
+        </is>
+      </c>
+      <c r="D72" s="8" t="inlineStr">
+        <is>
+          <t>inv.total</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="6" t="inlineStr">
+        <is>
+          <t>END:</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="1" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B76" s="1" t="inlineStr"/>
+      <c r="C76" s="1" t="inlineStr"/>
+      <c r="D76" s="1" t="inlineStr"/>
+      <c r="E76" s="1" t="inlineStr">
+        <is>
+          <t>── QUICK REFERENCE ──────────────────────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="1" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B77" s="1" t="inlineStr">
         <is>
           <t>doc: | free text</t>
         </is>
       </c>
-      <c r="C66" s="1" t="inlineStr"/>
-      <c r="D66" s="1" t="inlineStr">
+      <c r="C77" s="1" t="inlineStr"/>
+      <c r="D77" s="1" t="inlineStr">
         <is>
           <t>Inline comment. Ignored by engine.</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="3" t="inlineStr">
+    <row r="78">
+      <c r="A78" s="3" t="inlineStr">
         <is>
           <t>config:</t>
         </is>
       </c>
-      <c r="B67" s="3" t="inlineStr">
+      <c r="B78" s="3" t="inlineStr">
         <is>
           <t>config: | key | value</t>
         </is>
       </c>
-      <c r="C67" s="3" t="inlineStr"/>
-      <c r="D67" s="3" t="inlineStr">
+      <c r="C78" s="3" t="inlineStr"/>
+      <c r="D78" s="3" t="inlineStr">
         <is>
           <t>Global setting. Keys: read.direction, currency.sign, empty.aliases</t>
         </is>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" s="4" t="inlineStr">
+    <row r="79">
+      <c r="A79" s="4" t="inlineStr">
         <is>
           <t>lbl:</t>
         </is>
       </c>
-      <c r="B68" s="4" t="inlineStr">
+      <c r="B79" s="4" t="inlineStr">
         <is>
           <t>lbl: | name | type | regex</t>
         </is>
       </c>
-      <c r="C68" s="4" t="inlineStr"/>
-      <c r="D68" s="4" t="inlineStr">
+      <c r="C79" s="4" t="inlineStr"/>
+      <c r="D79" s="4" t="inlineStr">
         <is>
           <t>Anchor label. Matched but never in output.</t>
         </is>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" s="5" t="inlineStr">
+    <row r="80">
+      <c r="A80" s="5" t="inlineStr">
         <is>
           <t>var:</t>
         </is>
       </c>
-      <c r="B69" s="5" t="inlineStr">
+      <c r="B80" s="5" t="inlineStr">
         <is>
           <t>var: | name | type | regex</t>
         </is>
       </c>
-      <c r="C69" s="5" t="inlineStr"/>
-      <c r="D69" s="5" t="inlineStr">
+      <c r="C80" s="5" t="inlineStr"/>
+      <c r="D80" s="5" t="inlineStr">
         <is>
           <t>Extracted variable. Use dot notation for nesting.</t>
         </is>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
+    <row r="81">
+      <c r="A81" t="inlineStr">
         <is>
           <t>cell:next</t>
         </is>
       </c>
-      <c r="B70" t="inlineStr">
+      <c r="B81" t="inlineStr">
         <is>
           <t>cell:next | FieldName</t>
         </is>
       </c>
-      <c r="C70" t="inlineStr"/>
-      <c r="D70" t="inlineStr">
+      <c r="C81" t="inlineStr"/>
+      <c r="D81" t="inlineStr">
         <is>
           <t>Read next non-empty cell (alias: cell:1).</t>
         </is>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
+    <row r="82">
+      <c r="A82" t="inlineStr">
         <is>
           <t>cell:next</t>
         </is>
       </c>
-      <c r="B71" t="inlineStr">
+      <c r="B82" t="inlineStr">
         <is>
           <t>cell:next | IGNORE</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr"/>
-      <c r="D71" t="inlineStr">
+      <c r="C82" t="inlineStr"/>
+      <c r="D82" t="inlineStr">
         <is>
           <t>Skip next non-empty cell without capturing.</t>
         </is>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
+    <row r="83">
+      <c r="A83" t="inlineStr">
         <is>
           <t>cell:next</t>
         </is>
       </c>
-      <c r="B72" t="inlineStr">
+      <c r="B83" t="inlineStr">
         <is>
           <t>cell:B5 | FieldName</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr"/>
-      <c r="D72" t="inlineStr">
+      <c r="C83" t="inlineStr"/>
+      <c r="D83" t="inlineStr">
         <is>
           <t>Jump directly to B5 (absolute reference). Ordering must be forward.</t>
         </is>
       </c>
     </row>
-    <row r="73">
-      <c r="A73" s="7" t="inlineStr">
+    <row r="84">
+      <c r="A84" s="7" t="inlineStr">
         <is>
           <t>table:*</t>
         </is>
       </c>
-      <c r="B73" s="7" t="inlineStr">
+      <c r="B84" s="7" t="inlineStr">
         <is>
           <t>table:*  (or table:1)</t>
         </is>
       </c>
-      <c r="C73" s="7" t="inlineStr"/>
-      <c r="D73" s="7" t="inlineStr">
+      <c r="C84" s="7" t="inlineStr"/>
+      <c r="D84" s="7" t="inlineStr">
         <is>
           <t>Begin a repeating table block.</t>
         </is>
       </c>
     </row>
-    <row r="74">
-      <c r="A74" s="8" t="inlineStr">
+    <row r="85">
+      <c r="A85" s="8" t="inlineStr">
         <is>
           <t>HEADER:N</t>
         </is>
       </c>
-      <c r="B74" s="8" t="inlineStr">
+      <c r="B85" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve"> | HEADER:1 | F1 | F2</t>
         </is>
       </c>
-      <c r="C74" s="8" t="inlineStr"/>
-      <c r="D74" s="8" t="inlineStr">
+      <c r="C85" s="8" t="inlineStr"/>
+      <c r="D85" s="8" t="inlineStr">
         <is>
           <t>Strict header row template (col A must be blank).</t>
         </is>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" s="8" t="inlineStr">
+    <row r="86">
+      <c r="A86" s="8" t="inlineStr">
         <is>
           <t>DATA:*</t>
         </is>
       </c>
-      <c r="B75" s="8" t="inlineStr">
+      <c r="B86" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve"> | DATA:* | F1 | F2</t>
         </is>
       </c>
-      <c r="C75" s="8" t="inlineStr"/>
-      <c r="D75" s="8" t="inlineStr">
-        <is>
-          <t>Data row template (lenient validation).</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="8" t="inlineStr">
+      <c r="C86" s="8" t="inlineStr"/>
+      <c r="D86" s="8" t="inlineStr">
+        <is>
+          <t>Data row template (greedy, lenient validation).</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="8" t="inlineStr">
+        <is>
+          <t>DATA:{n,m}</t>
+        </is>
+      </c>
+      <c r="B87" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> | DATA:{0,15} | F1 | F2</t>
+        </is>
+      </c>
+      <c r="C87" s="8" t="inlineStr"/>
+      <c r="D87" s="8" t="inlineStr">
+        <is>
+          <t>Bounded data: scan at most m physical rows, warn if &lt; n.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>SKIP_IF</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> | SKIP_IF | EMPTY | IGNORE</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr"/>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Skip row if non-IGNORE columns match. Only with DATA:{n,m}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="8" t="inlineStr">
         <is>
           <t>FOOTER:N</t>
         </is>
       </c>
-      <c r="B76" s="8" t="inlineStr">
+      <c r="B89" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve"> | FOOTER:1 | F1 | F2</t>
         </is>
       </c>
-      <c r="C76" s="8" t="inlineStr"/>
-      <c r="D76" s="8" t="inlineStr">
+      <c r="C89" s="8" t="inlineStr"/>
+      <c r="D89" s="8" t="inlineStr">
         <is>
           <t>Strict footer row template.</t>
         </is>
       </c>
     </row>
-    <row r="77">
-      <c r="A77" s="8" t="inlineStr">
+    <row r="90">
+      <c r="A90" s="8" t="inlineStr">
         <is>
           <t>SPLITTER</t>
         </is>
       </c>
-      <c r="B77" s="8" t="inlineStr">
+      <c r="B90" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve"> | SPLITTER:1</t>
         </is>
       </c>
-      <c r="C77" s="8" t="inlineStr"/>
-      <c r="D77" s="8" t="inlineStr">
+      <c r="C90" s="8" t="inlineStr"/>
+      <c r="D90" s="8" t="inlineStr">
         <is>
           <t>All columns must be blank (separator row).</t>
         </is>

</xml_diff>

<commit_message>
Add '#' trailing comments to pattern files
A cell whose text starts with '#' is a comment running to the end of that row,
allowed as a TRAILING annotation on config:/var:/def:/lbl:/cell:/START: rows
(after the row's real columns: var/lbl → col E+, cell → C+, config → D+,
START → B+). doc:/info: remain whole-line comment rows.

Rules:
- A '#' in a value column (e.g. a regex `#\d+` in col D) stays a value — comments
  only live after the meaningful columns.
- table:/HEADER:/DATA:/FOOTER: rows get NO comment processing; '#' is literal there.
- Fail fast: non-empty, non-'#' content in a comment position raises PatternError
  (catches a value typed into the wrong column instead of silently dropping it).

Parser: new _check_comment_zone() wired into the relevant branches. Tests:
TestPatternComments (9). Docs: a Comments section in docs/pattern-file.md and
explanatory rows in the generated pattern-reference.xlsx. Full suite: 939 passed.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/pattern-reference.xlsx
+++ b/docs/pattern-reference.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F91"/>
+  <dimension ref="A1:F94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -934,79 +934,47 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="5" t="inlineStr">
-        <is>
-          <t>var:</t>
-        </is>
-      </c>
-      <c r="B30" s="5" t="inlineStr">
-        <is>
-          <t>po.number</t>
-        </is>
-      </c>
-      <c r="C30" s="5" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="D30" s="5" t="inlineStr">
-        <is>
-          <t>PO-[0-9]{4}</t>
-        </is>
-      </c>
-      <c r="E30" s="5" t="inlineStr">
-        <is>
-          <t>Matches e.g. "PO-2026". Output key: {"po": {"number": ...}}</t>
+      <c r="A30" s="1" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B30" s="1" t="inlineStr"/>
+      <c r="C30" s="1" t="inlineStr"/>
+      <c r="D30" s="1" t="inlineStr"/>
+      <c r="E30" s="1" t="inlineStr">
+        <is>
+          <t>Comments: a doc:/info: row is a whole-line comment. On config/var/lbl/cell/START rows,</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="5" t="inlineStr">
-        <is>
-          <t>var:</t>
-        </is>
-      </c>
-      <c r="B31" s="5" t="inlineStr">
-        <is>
-          <t>po.date</t>
-        </is>
-      </c>
-      <c r="C31" s="5" t="inlineStr">
-        <is>
-          <t>date</t>
-        </is>
-      </c>
-      <c r="D31" s="5" t="inlineStr"/>
-      <c r="E31" s="5" t="inlineStr">
-        <is>
-          <t>Any date cell. Leave regex empty for date/datetime.</t>
+      <c r="A31" s="1" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B31" s="1" t="inlineStr"/>
+      <c r="C31" s="1" t="inlineStr"/>
+      <c r="D31" s="1" t="inlineStr"/>
+      <c r="E31" s="1" t="inlineStr">
+        <is>
+          <t>a cell starting with # AFTER the real columns is a trailing comment to end of row</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="5" t="inlineStr">
-        <is>
-          <t>var:</t>
-        </is>
-      </c>
-      <c r="B32" s="5" t="inlineStr">
-        <is>
-          <t>vendor.name</t>
-        </is>
-      </c>
-      <c r="C32" s="5" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="D32" s="5" t="inlineStr">
-        <is>
-          <t>.+</t>
-        </is>
-      </c>
-      <c r="E32" s="5" t="inlineStr">
-        <is>
-          <t>Any non-empty string.</t>
+      <c r="A32" s="1" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B32" s="1" t="inlineStr"/>
+      <c r="C32" s="1" t="inlineStr"/>
+      <c r="D32" s="1" t="inlineStr"/>
+      <c r="E32" s="1" t="inlineStr">
+        <is>
+          <t>(var:/lbl: → col E+, cell: → col C+, config: → col D+). NOT in table: rows (# is literal there).</t>
         </is>
       </c>
     </row>
@@ -1018,7 +986,7 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>line.item</t>
+          <t>po.number</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
@@ -1028,12 +996,12 @@
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>.+</t>
+          <t>PO-[0-9]{4}</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>Table DATA field. Group prefix "line" → {"line": [...]}</t>
+          <t>Matches e.g. "PO-2026". Output key: {"po": {"number": ...}}</t>
         </is>
       </c>
     </row>
@@ -1045,22 +1013,18 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>line.qty</t>
+          <t>po.date</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>integer</t>
-        </is>
-      </c>
-      <c r="D34" s="5" t="inlineStr">
-        <is>
-          <t>[1-9][0-9]*</t>
-        </is>
-      </c>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr"/>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>Positive integer.</t>
+          <t>Any date cell. Leave regex empty for date/datetime.</t>
         </is>
       </c>
     </row>
@@ -1072,22 +1036,22 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>line.price</t>
+          <t>vendor.name</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>currency</t>
+          <t>string</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>.*</t>
+          <t>.+</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>Any currency value.</t>
+          <t>Any non-empty string.</t>
         </is>
       </c>
     </row>
@@ -1099,22 +1063,22 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>line.total</t>
+          <t>line.item</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>currency</t>
+          <t>string</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>.*</t>
+          <t>.+</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>Any currency value.</t>
+          <t>Table DATA field. Group prefix "line" → {"line": [...]}</t>
         </is>
       </c>
     </row>
@@ -1126,22 +1090,22 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>footer.label</t>
+          <t>line.qty</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>Grand Total</t>
+          <t>[1-9][0-9]*</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>FOOTER field — matches the literal "Grand Total".</t>
+          <t>Positive integer.</t>
         </is>
       </c>
     </row>
@@ -1153,67 +1117,103 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
+          <t>line.price</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>currency</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>.*</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>Any currency value.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>var:</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>line.total</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>currency</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>.*</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>Any currency value.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>var:</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>footer.label</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>Grand Total</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>FOOTER field — matches the literal "Grand Total".</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>var:</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
           <t>footer.value</t>
         </is>
       </c>
-      <c r="C38" s="5" t="inlineStr">
+      <c r="C41" s="5" t="inlineStr">
         <is>
           <t>currency</t>
         </is>
       </c>
-      <c r="D38" s="5" t="inlineStr">
+      <c r="D41" s="5" t="inlineStr">
         <is>
           <t>.*</t>
         </is>
       </c>
-      <c r="E38" s="5" t="inlineStr">
+      <c r="E41" s="5" t="inlineStr">
         <is>
           <t>FOOTER value field.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="1" t="inlineStr">
-        <is>
-          <t>doc:</t>
-        </is>
-      </c>
-      <c r="B40" s="1" t="inlineStr"/>
-      <c r="C40" s="1" t="inlineStr"/>
-      <c r="D40" s="1" t="inlineStr"/>
-      <c r="E40" s="1" t="inlineStr">
-        <is>
-          <t>Everything between START: and END: defines the extraction order.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="1" t="inlineStr">
-        <is>
-          <t>doc:</t>
-        </is>
-      </c>
-      <c r="B41" s="1" t="inlineStr"/>
-      <c r="C41" s="1" t="inlineStr"/>
-      <c r="D41" s="1" t="inlineStr"/>
-      <c r="E41" s="1" t="inlineStr">
-        <is>
-          <t>cell:next  reads the next non-empty cell (alias: cell:1). Scans in read.direction order.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="1" t="inlineStr">
-        <is>
-          <t>doc:</t>
-        </is>
-      </c>
-      <c r="B42" s="1" t="inlineStr"/>
-      <c r="C42" s="1" t="inlineStr"/>
-      <c r="D42" s="1" t="inlineStr"/>
-      <c r="E42" s="1" t="inlineStr">
-        <is>
-          <t>cell:B5    jumps directly to cell B5 (absolute A1-notation reference).</t>
         </is>
       </c>
     </row>
@@ -1228,90 +1228,78 @@
       <c r="D43" s="1" t="inlineStr"/>
       <c r="E43" s="1" t="inlineStr">
         <is>
+          <t>Everything between START: and END: defines the extraction order.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="1" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B44" s="1" t="inlineStr"/>
+      <c r="C44" s="1" t="inlineStr"/>
+      <c r="D44" s="1" t="inlineStr"/>
+      <c r="E44" s="1" t="inlineStr">
+        <is>
+          <t>cell:next  reads the next non-empty cell (alias: cell:1). Scans in read.direction order.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B45" s="1" t="inlineStr"/>
+      <c r="C45" s="1" t="inlineStr"/>
+      <c r="D45" s="1" t="inlineStr"/>
+      <c r="E45" s="1" t="inlineStr">
+        <is>
+          <t>cell:B5    jumps directly to cell B5 (absolute A1-notation reference).</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="1" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B46" s="1" t="inlineStr"/>
+      <c r="C46" s="1" t="inlineStr"/>
+      <c r="D46" s="1" t="inlineStr"/>
+      <c r="E46" s="1" t="inlineStr">
+        <is>
           <t>table:*    finds all instances of a repeating table block.</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="6" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="6" t="inlineStr">
         <is>
           <t>START:</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="7" t="inlineStr">
-        <is>
-          <t>cell:A1</t>
-        </is>
-      </c>
-      <c r="B45" s="7" t="inlineStr">
-        <is>
-          <t>po_label</t>
-        </is>
-      </c>
-      <c r="C45" s="7" t="inlineStr"/>
-      <c r="D45" s="7" t="inlineStr"/>
-      <c r="E45" s="7" t="inlineStr">
-        <is>
-          <t>Jump to A1 and read "PO Number:" anchor (lbl: field — not in output).</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="7" t="inlineStr">
-        <is>
-          <t>cell:next</t>
-        </is>
-      </c>
-      <c r="B46" s="7" t="inlineStr">
-        <is>
-          <t>po.number</t>
-        </is>
-      </c>
-      <c r="C46" s="7" t="inlineStr"/>
-      <c r="D46" s="7" t="inlineStr"/>
-      <c r="E46" s="7" t="inlineStr">
-        <is>
-          <t>Read next non-empty cell after A1 → the PO number.</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="7" t="inlineStr">
-        <is>
-          <t>cell:C1</t>
-        </is>
-      </c>
-      <c r="B47" s="7" t="inlineStr">
-        <is>
-          <t>date_label</t>
-        </is>
-      </c>
-      <c r="C47" s="7" t="inlineStr"/>
-      <c r="D47" s="7" t="inlineStr"/>
-      <c r="E47" s="7" t="inlineStr">
-        <is>
-          <t>Jump to C1 and read "Date:" anchor.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
         <is>
-          <t>cell:next</t>
+          <t>cell:A1</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>po.date</t>
+          <t>po_label</t>
         </is>
       </c>
       <c r="C48" s="7" t="inlineStr"/>
       <c r="D48" s="7" t="inlineStr"/>
       <c r="E48" s="7" t="inlineStr">
         <is>
-          <t>Read next non-empty cell after C1 → the PO date.</t>
+          <t>Jump to A1 and read "PO Number:" anchor (lbl: field — not in output).</t>
         </is>
       </c>
     </row>
@@ -1323,48 +1311,52 @@
       </c>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>vendor_label</t>
+          <t>po.number</t>
         </is>
       </c>
       <c r="C49" s="7" t="inlineStr"/>
       <c r="D49" s="7" t="inlineStr"/>
       <c r="E49" s="7" t="inlineStr">
         <is>
-          <t>Read next non-empty cell → "Vendor:" anchor.</t>
+          <t>Read next non-empty cell after A1 → the PO number.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
         <is>
-          <t>cell:next</t>
+          <t>cell:C1</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>vendor.name</t>
+          <t>date_label</t>
         </is>
       </c>
       <c r="C50" s="7" t="inlineStr"/>
       <c r="D50" s="7" t="inlineStr"/>
       <c r="E50" s="7" t="inlineStr">
         <is>
-          <t>Extract the vendor name.</t>
+          <t>Jump to C1 and read "Date:" anchor.</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="1" t="inlineStr">
-        <is>
-          <t>doc:</t>
-        </is>
-      </c>
-      <c r="B51" s="1" t="inlineStr"/>
-      <c r="C51" s="1" t="inlineStr"/>
-      <c r="D51" s="1" t="inlineStr"/>
-      <c r="E51" s="1" t="inlineStr">
-        <is>
-          <t>Use IGNORE to skip a non-empty cell without defining a field for it.</t>
+      <c r="A51" s="7" t="inlineStr">
+        <is>
+          <t>cell:next</t>
+        </is>
+      </c>
+      <c r="B51" s="7" t="inlineStr">
+        <is>
+          <t>po.date</t>
+        </is>
+      </c>
+      <c r="C51" s="7" t="inlineStr"/>
+      <c r="D51" s="7" t="inlineStr"/>
+      <c r="E51" s="7" t="inlineStr">
+        <is>
+          <t>Read next non-empty cell after C1 → the PO date.</t>
         </is>
       </c>
     </row>
@@ -1376,14 +1368,33 @@
       </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>IGNORE</t>
+          <t>vendor_label</t>
         </is>
       </c>
       <c r="C52" s="7" t="inlineStr"/>
       <c r="D52" s="7" t="inlineStr"/>
       <c r="E52" s="7" t="inlineStr">
         <is>
-          <t>Skip one non-empty cell without capturing it.</t>
+          <t>Read next non-empty cell → "Vendor:" anchor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="7" t="inlineStr">
+        <is>
+          <t>cell:next</t>
+        </is>
+      </c>
+      <c r="B53" s="7" t="inlineStr">
+        <is>
+          <t>vendor.name</t>
+        </is>
+      </c>
+      <c r="C53" s="7" t="inlineStr"/>
+      <c r="D53" s="7" t="inlineStr"/>
+      <c r="E53" s="7" t="inlineStr">
+        <is>
+          <t>Extract the vendor name.</t>
         </is>
       </c>
     </row>
@@ -1398,158 +1409,147 @@
       <c r="D54" s="1" t="inlineStr"/>
       <c r="E54" s="1" t="inlineStr">
         <is>
+          <t>Use IGNORE to skip a non-empty cell without defining a field for it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="7" t="inlineStr">
+        <is>
+          <t>cell:next</t>
+        </is>
+      </c>
+      <c r="B55" s="7" t="inlineStr">
+        <is>
+          <t>IGNORE</t>
+        </is>
+      </c>
+      <c r="C55" s="7" t="inlineStr"/>
+      <c r="D55" s="7" t="inlineStr"/>
+      <c r="E55" s="7" t="inlineStr">
+        <is>
+          <t>Skip one non-empty cell without capturing it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="1" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B57" s="1" t="inlineStr"/>
+      <c r="C57" s="1" t="inlineStr"/>
+      <c r="D57" s="1" t="inlineStr"/>
+      <c r="E57" s="1" t="inlineStr">
+        <is>
           <t>table:* matches 0-or-more mini-table instances in greedy order.</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="1" t="inlineStr">
-        <is>
-          <t>doc:</t>
-        </is>
-      </c>
-      <c r="B55" s="1" t="inlineStr"/>
-      <c r="C55" s="1" t="inlineStr"/>
-      <c r="D55" s="1" t="inlineStr"/>
-      <c r="E55" s="1" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="1" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B58" s="1" t="inlineStr"/>
+      <c r="C58" s="1" t="inlineStr"/>
+      <c r="D58" s="1" t="inlineStr"/>
+      <c r="E58" s="1" t="inlineStr">
         <is>
           <t>Use table:1 when exactly one instance is expected.</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="7" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="7" t="inlineStr">
         <is>
           <t>table:*</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="8" t="n"/>
-      <c r="B57" s="8" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="8" t="n"/>
+      <c r="B60" s="8" t="inlineStr">
         <is>
           <t>HEADER:1</t>
         </is>
       </c>
-      <c r="C57" s="8" t="inlineStr">
+      <c r="C60" s="8" t="inlineStr">
         <is>
           <t>col_item</t>
         </is>
       </c>
-      <c r="D57" s="8" t="inlineStr">
+      <c r="D60" s="8" t="inlineStr">
         <is>
           <t>col_qty</t>
         </is>
       </c>
-      <c r="E57" s="8" t="inlineStr">
+      <c r="E60" s="8" t="inlineStr">
         <is>
           <t>col_price</t>
         </is>
       </c>
-      <c r="F57" s="8" t="inlineStr">
+      <c r="F60" s="8" t="inlineStr">
         <is>
           <t>col_total</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="8" t="n"/>
-      <c r="B58" s="8" t="inlineStr">
+    <row r="61">
+      <c r="A61" s="8" t="n"/>
+      <c r="B61" s="8" t="inlineStr">
         <is>
           <t>DATA:*</t>
         </is>
       </c>
-      <c r="C58" s="8" t="inlineStr">
+      <c r="C61" s="8" t="inlineStr">
         <is>
           <t>line.item</t>
         </is>
       </c>
-      <c r="D58" s="8" t="inlineStr">
+      <c r="D61" s="8" t="inlineStr">
         <is>
           <t>line.qty</t>
         </is>
       </c>
-      <c r="E58" s="8" t="inlineStr">
+      <c r="E61" s="8" t="inlineStr">
         <is>
           <t>line.price</t>
         </is>
       </c>
-      <c r="F58" s="8" t="inlineStr">
+      <c r="F61" s="8" t="inlineStr">
         <is>
           <t>line.total</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="8" t="n"/>
-      <c r="B59" s="8" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="8" t="n"/>
+      <c r="B62" s="8" t="inlineStr">
         <is>
           <t>FOOTER:1</t>
         </is>
       </c>
-      <c r="C59" s="8" t="inlineStr">
+      <c r="C62" s="8" t="inlineStr">
         <is>
           <t>footer.label</t>
         </is>
       </c>
-      <c r="D59" s="8" t="inlineStr">
+      <c r="D62" s="8" t="inlineStr">
         <is>
           <t>IGNORE</t>
         </is>
       </c>
-      <c r="E59" s="8" t="inlineStr">
+      <c r="E62" s="8" t="inlineStr">
         <is>
           <t>IGNORE</t>
         </is>
       </c>
-      <c r="F59" s="8" t="inlineStr">
+      <c r="F62" s="8" t="inlineStr">
         <is>
           <t>footer.value</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="1" t="inlineStr">
-        <is>
-          <t>doc:</t>
-        </is>
-      </c>
-      <c r="B60" s="1" t="inlineStr"/>
-      <c r="C60" s="1" t="inlineStr"/>
-      <c r="D60" s="1" t="inlineStr"/>
-      <c r="E60" s="1" t="inlineStr">
-        <is>
-          <t>HEADER/FOOTER are strict: wrong or missing value = no match.</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="1" t="inlineStr">
-        <is>
-          <t>doc:</t>
-        </is>
-      </c>
-      <c r="B61" s="1" t="inlineStr"/>
-      <c r="C61" s="1" t="inlineStr"/>
-      <c r="D61" s="1" t="inlineStr"/>
-      <c r="E61" s="1" t="inlineStr">
-        <is>
-          <t>DATA rows are lenient: wrong value emits a warning but extraction continues.</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="1" t="inlineStr">
-        <is>
-          <t>doc:</t>
-        </is>
-      </c>
-      <c r="B62" s="1" t="inlineStr"/>
-      <c r="C62" s="1" t="inlineStr"/>
-      <c r="D62" s="1" t="inlineStr"/>
-      <c r="E62" s="1" t="inlineStr">
-        <is>
-          <t>EMPTY column keyword: cell must be blank. IGNORE: consume without matching.</t>
         </is>
       </c>
     </row>
@@ -1564,7 +1564,7 @@
       <c r="D63" s="1" t="inlineStr"/>
       <c r="E63" s="1" t="inlineStr">
         <is>
-          <t>── BOUNDED DATA + SKIP_IF (fixed-slot templates) ───────────────────────</t>
+          <t>HEADER/FOOTER are strict: wrong or missing value = no match.</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="D64" s="1" t="inlineStr"/>
       <c r="E64" s="1" t="inlineStr">
         <is>
-          <t>Use DATA:{n,m} when the template pre-allocates a fixed number of rows.</t>
+          <t>DATA rows are lenient: wrong value emits a warning but extraction continues.</t>
         </is>
       </c>
     </row>
@@ -1594,7 +1594,7 @@
       <c r="D65" s="1" t="inlineStr"/>
       <c r="E65" s="1" t="inlineStr">
         <is>
-          <t>n = min total physical rows expected, m = max total rows to scan.</t>
+          <t>EMPTY column keyword: cell must be blank. IGNORE: consume without matching.</t>
         </is>
       </c>
     </row>
@@ -1609,7 +1609,7 @@
       <c r="D66" s="1" t="inlineStr"/>
       <c r="E66" s="1" t="inlineStr">
         <is>
-          <t>SKIP_IF: rows matching the condition are silently excluded from output</t>
+          <t>── BOUNDED DATA + SKIP_IF (fixed-slot templates) ───────────────────────</t>
         </is>
       </c>
     </row>
@@ -1624,7 +1624,7 @@
       <c r="D67" s="1" t="inlineStr"/>
       <c r="E67" s="1" t="inlineStr">
         <is>
-          <t>but still count toward the {n,m} bounds.</t>
+          <t>Use DATA:{n,m} when the template pre-allocates a fixed number of rows.</t>
         </is>
       </c>
     </row>
@@ -1639,68 +1639,59 @@
       <c r="D68" s="1" t="inlineStr"/>
       <c r="E68" s="1" t="inlineStr">
         <is>
+          <t>n = min total physical rows expected, m = max total rows to scan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="1" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B69" s="1" t="inlineStr"/>
+      <c r="C69" s="1" t="inlineStr"/>
+      <c r="D69" s="1" t="inlineStr"/>
+      <c r="E69" s="1" t="inlineStr">
+        <is>
+          <t>SKIP_IF: rows matching the condition are silently excluded from output</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="1" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B70" s="1" t="inlineStr"/>
+      <c r="C70" s="1" t="inlineStr"/>
+      <c r="D70" s="1" t="inlineStr"/>
+      <c r="E70" s="1" t="inlineStr">
+        <is>
+          <t>but still count toward the {n,m} bounds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="1" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B71" s="1" t="inlineStr"/>
+      <c r="C71" s="1" t="inlineStr"/>
+      <c r="D71" s="1" t="inlineStr"/>
+      <c r="E71" s="1" t="inlineStr">
+        <is>
           <t>SKIP_IF is only valid with DATA:{n,m}.</t>
         </is>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" s="7" t="inlineStr">
+    <row r="72">
+      <c r="A72" s="7" t="inlineStr">
         <is>
           <t>table:1</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="8" t="n"/>
-      <c r="B70" s="8" t="inlineStr">
-        <is>
-          <t>HEADER:1</t>
-        </is>
-      </c>
-      <c r="C70" s="8" t="inlineStr">
-        <is>
-          <t>col_item</t>
-        </is>
-      </c>
-      <c r="D70" s="8" t="inlineStr">
-        <is>
-          <t>col_qty</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="8" t="n"/>
-      <c r="B71" s="8" t="inlineStr">
-        <is>
-          <t>SKIP_IF</t>
-        </is>
-      </c>
-      <c r="C71" s="8" t="inlineStr">
-        <is>
-          <t>EMPTY</t>
-        </is>
-      </c>
-      <c r="D71" s="8" t="inlineStr">
-        <is>
-          <t>IGNORE</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="8" t="n"/>
-      <c r="B72" s="8" t="inlineStr">
-        <is>
-          <t>DATA:{0,15}</t>
-        </is>
-      </c>
-      <c r="C72" s="8" t="inlineStr">
-        <is>
-          <t>line.item</t>
-        </is>
-      </c>
-      <c r="D72" s="8" t="inlineStr">
-        <is>
-          <t>line.qty</t>
         </is>
       </c>
     </row>
@@ -1708,289 +1699,343 @@
       <c r="A73" s="8" t="n"/>
       <c r="B73" s="8" t="inlineStr">
         <is>
+          <t>HEADER:1</t>
+        </is>
+      </c>
+      <c r="C73" s="8" t="inlineStr">
+        <is>
+          <t>col_item</t>
+        </is>
+      </c>
+      <c r="D73" s="8" t="inlineStr">
+        <is>
+          <t>col_qty</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="8" t="n"/>
+      <c r="B74" s="8" t="inlineStr">
+        <is>
+          <t>SKIP_IF</t>
+        </is>
+      </c>
+      <c r="C74" s="8" t="inlineStr">
+        <is>
+          <t>EMPTY</t>
+        </is>
+      </c>
+      <c r="D74" s="8" t="inlineStr">
+        <is>
+          <t>IGNORE</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="8" t="n"/>
+      <c r="B75" s="8" t="inlineStr">
+        <is>
+          <t>DATA:{0,15}</t>
+        </is>
+      </c>
+      <c r="C75" s="8" t="inlineStr">
+        <is>
+          <t>line.item</t>
+        </is>
+      </c>
+      <c r="D75" s="8" t="inlineStr">
+        <is>
+          <t>line.qty</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="8" t="n"/>
+      <c r="B76" s="8" t="inlineStr">
+        <is>
           <t>FOOTER:1</t>
         </is>
       </c>
-      <c r="C73" s="8" t="inlineStr">
+      <c r="C76" s="8" t="inlineStr">
         <is>
           <t>lbl_total</t>
         </is>
       </c>
-      <c r="D73" s="8" t="inlineStr">
+      <c r="D76" s="8" t="inlineStr">
         <is>
           <t>inv.total</t>
         </is>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" s="6" t="inlineStr">
+    <row r="78">
+      <c r="A78" s="6" t="inlineStr">
         <is>
           <t>END:</t>
         </is>
       </c>
     </row>
-    <row r="77">
-      <c r="A77" s="1" t="inlineStr">
-        <is>
-          <t>doc:</t>
-        </is>
-      </c>
-      <c r="B77" s="1" t="inlineStr"/>
-      <c r="C77" s="1" t="inlineStr"/>
-      <c r="D77" s="1" t="inlineStr"/>
-      <c r="E77" s="1" t="inlineStr">
+    <row r="80">
+      <c r="A80" s="1" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B80" s="1" t="inlineStr"/>
+      <c r="C80" s="1" t="inlineStr"/>
+      <c r="D80" s="1" t="inlineStr"/>
+      <c r="E80" s="1" t="inlineStr">
         <is>
           <t>── QUICK REFERENCE ──────────────────────────────────────────────</t>
         </is>
       </c>
     </row>
-    <row r="78">
-      <c r="A78" s="1" t="inlineStr">
-        <is>
-          <t>doc:</t>
-        </is>
-      </c>
-      <c r="B78" s="1" t="inlineStr">
+    <row r="81">
+      <c r="A81" s="1" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B81" s="1" t="inlineStr">
         <is>
           <t>doc: | free text</t>
         </is>
       </c>
-      <c r="C78" s="1" t="inlineStr"/>
-      <c r="D78" s="1" t="inlineStr">
+      <c r="C81" s="1" t="inlineStr"/>
+      <c r="D81" s="1" t="inlineStr">
         <is>
           <t>Inline comment. Ignored by engine.</t>
         </is>
       </c>
     </row>
-    <row r="79">
-      <c r="A79" s="3" t="inlineStr">
+    <row r="82">
+      <c r="A82" s="3" t="inlineStr">
         <is>
           <t>config:</t>
         </is>
       </c>
-      <c r="B79" s="3" t="inlineStr">
+      <c r="B82" s="3" t="inlineStr">
         <is>
           <t>config: | key | value</t>
         </is>
       </c>
-      <c r="C79" s="3" t="inlineStr"/>
-      <c r="D79" s="3" t="inlineStr">
+      <c r="C82" s="3" t="inlineStr"/>
+      <c r="D82" s="3" t="inlineStr">
         <is>
           <t>Global setting. Keys: read.direction, currency.sign, empty.aliases, ignore.case</t>
         </is>
       </c>
     </row>
-    <row r="80">
-      <c r="A80" s="4" t="inlineStr">
+    <row r="83">
+      <c r="A83" s="4" t="inlineStr">
         <is>
           <t>lbl:</t>
         </is>
       </c>
-      <c r="B80" s="4" t="inlineStr">
+      <c r="B83" s="4" t="inlineStr">
         <is>
           <t>lbl: | name | type | regex</t>
         </is>
       </c>
-      <c r="C80" s="4" t="inlineStr"/>
-      <c r="D80" s="4" t="inlineStr">
+      <c r="C83" s="4" t="inlineStr"/>
+      <c r="D83" s="4" t="inlineStr">
         <is>
           <t>Anchor label. Matched but never in output.</t>
         </is>
       </c>
     </row>
-    <row r="81">
-      <c r="A81" s="5" t="inlineStr">
+    <row r="84">
+      <c r="A84" s="5" t="inlineStr">
         <is>
           <t>var:</t>
         </is>
       </c>
-      <c r="B81" s="5" t="inlineStr">
+      <c r="B84" s="5" t="inlineStr">
         <is>
           <t>var: | name | type | regex</t>
         </is>
       </c>
-      <c r="C81" s="5" t="inlineStr"/>
-      <c r="D81" s="5" t="inlineStr">
+      <c r="C84" s="5" t="inlineStr"/>
+      <c r="D84" s="5" t="inlineStr">
         <is>
           <t>Extracted variable. Use dot notation for nesting.</t>
         </is>
       </c>
     </row>
-    <row r="82">
-      <c r="A82" t="inlineStr">
+    <row r="85">
+      <c r="A85" t="inlineStr">
         <is>
           <t>cell:next</t>
         </is>
       </c>
-      <c r="B82" t="inlineStr">
+      <c r="B85" t="inlineStr">
         <is>
           <t>cell:next | FieldName</t>
         </is>
       </c>
-      <c r="C82" t="inlineStr"/>
-      <c r="D82" t="inlineStr">
+      <c r="C85" t="inlineStr"/>
+      <c r="D85" t="inlineStr">
         <is>
           <t>Read next non-empty cell (alias: cell:1).</t>
         </is>
       </c>
     </row>
-    <row r="83">
-      <c r="A83" t="inlineStr">
+    <row r="86">
+      <c r="A86" t="inlineStr">
         <is>
           <t>cell:next</t>
         </is>
       </c>
-      <c r="B83" t="inlineStr">
+      <c r="B86" t="inlineStr">
         <is>
           <t>cell:next | IGNORE</t>
         </is>
       </c>
-      <c r="C83" t="inlineStr"/>
-      <c r="D83" t="inlineStr">
+      <c r="C86" t="inlineStr"/>
+      <c r="D86" t="inlineStr">
         <is>
           <t>Skip next non-empty cell without capturing.</t>
         </is>
       </c>
     </row>
-    <row r="84">
-      <c r="A84" t="inlineStr">
+    <row r="87">
+      <c r="A87" t="inlineStr">
         <is>
           <t>cell:next</t>
         </is>
       </c>
-      <c r="B84" t="inlineStr">
+      <c r="B87" t="inlineStr">
         <is>
           <t>cell:B5 | FieldName</t>
         </is>
       </c>
-      <c r="C84" t="inlineStr"/>
-      <c r="D84" t="inlineStr">
+      <c r="C87" t="inlineStr"/>
+      <c r="D87" t="inlineStr">
         <is>
           <t>Jump directly to B5 (absolute reference). Ordering must be forward.</t>
         </is>
       </c>
     </row>
-    <row r="85">
-      <c r="A85" s="7" t="inlineStr">
+    <row r="88">
+      <c r="A88" s="7" t="inlineStr">
         <is>
           <t>table:*</t>
         </is>
       </c>
-      <c r="B85" s="7" t="inlineStr">
+      <c r="B88" s="7" t="inlineStr">
         <is>
           <t>table:*  (or table:1)</t>
         </is>
       </c>
-      <c r="C85" s="7" t="inlineStr"/>
-      <c r="D85" s="7" t="inlineStr">
+      <c r="C88" s="7" t="inlineStr"/>
+      <c r="D88" s="7" t="inlineStr">
         <is>
           <t>Begin a repeating table block.</t>
         </is>
       </c>
     </row>
-    <row r="86">
-      <c r="A86" s="8" t="inlineStr">
+    <row r="89">
+      <c r="A89" s="8" t="inlineStr">
         <is>
           <t>HEADER:N</t>
         </is>
       </c>
-      <c r="B86" s="8" t="inlineStr">
+      <c r="B89" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve"> | HEADER:1 | F1 | F2</t>
         </is>
       </c>
-      <c r="C86" s="8" t="inlineStr"/>
-      <c r="D86" s="8" t="inlineStr">
+      <c r="C89" s="8" t="inlineStr"/>
+      <c r="D89" s="8" t="inlineStr">
         <is>
           <t>Strict header row template (col A must be blank).</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" s="8" t="inlineStr">
-        <is>
-          <t>DATA:*</t>
-        </is>
-      </c>
-      <c r="B87" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> | DATA:* | F1 | F2</t>
-        </is>
-      </c>
-      <c r="C87" s="8" t="inlineStr"/>
-      <c r="D87" s="8" t="inlineStr">
-        <is>
-          <t>Data row template (greedy, lenient validation).</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" s="8" t="inlineStr">
-        <is>
-          <t>DATA:{n,m}</t>
-        </is>
-      </c>
-      <c r="B88" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> | DATA:{0,15} | F1 | F2</t>
-        </is>
-      </c>
-      <c r="C88" s="8" t="inlineStr"/>
-      <c r="D88" s="8" t="inlineStr">
-        <is>
-          <t>Bounded data: scan at most m physical rows, warn if &lt; n.</t>
-        </is>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" t="inlineStr">
-        <is>
-          <t>SKIP_IF</t>
-        </is>
-      </c>
-      <c r="B89" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> | SKIP_IF | EMPTY | IGNORE</t>
-        </is>
-      </c>
-      <c r="C89" t="inlineStr"/>
-      <c r="D89" t="inlineStr">
-        <is>
-          <t>Skip row if non-IGNORE columns match. Only with DATA:{n,m}.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="8" t="inlineStr">
         <is>
-          <t>FOOTER:N</t>
+          <t>DATA:*</t>
         </is>
       </c>
       <c r="B90" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | FOOTER:1 | F1 | F2</t>
+          <t xml:space="preserve"> | DATA:* | F1 | F2</t>
         </is>
       </c>
       <c r="C90" s="8" t="inlineStr"/>
       <c r="D90" s="8" t="inlineStr">
         <is>
-          <t>Strict footer row template.</t>
+          <t>Data row template (greedy, lenient validation).</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="8" t="inlineStr">
         <is>
-          <t>SPLITTER</t>
+          <t>DATA:{n,m}</t>
         </is>
       </c>
       <c r="B91" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | SPLITTER:1</t>
+          <t xml:space="preserve"> | DATA:{0,15} | F1 | F2</t>
         </is>
       </c>
       <c r="C91" s="8" t="inlineStr"/>
       <c r="D91" s="8" t="inlineStr">
+        <is>
+          <t>Bounded data: scan at most m physical rows, warn if &lt; n.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>SKIP_IF</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> | SKIP_IF | EMPTY | IGNORE</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr"/>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Skip row if non-IGNORE columns match. Only with DATA:{n,m}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="8" t="inlineStr">
+        <is>
+          <t>FOOTER:N</t>
+        </is>
+      </c>
+      <c r="B93" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> | FOOTER:1 | F1 | F2</t>
+        </is>
+      </c>
+      <c r="C93" s="8" t="inlineStr"/>
+      <c r="D93" s="8" t="inlineStr">
+        <is>
+          <t>Strict footer row template.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="8" t="inlineStr">
+        <is>
+          <t>SPLITTER</t>
+        </is>
+      </c>
+      <c r="B94" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> | SPLITTER:1</t>
+        </is>
+      </c>
+      <c r="C94" s="8" t="inlineStr"/>
+      <c r="D94" s="8" t="inlineStr">
         <is>
           <t>All columns must be blank (separator row).</t>
         </is>

</xml_diff>

<commit_message>
docs: regenerate pattern-reference.xlsx (seek: + SKIP_IF updates)
Adds the seek: quick-reference row and updates the SKIP_IF description
to reflect that it is now valid with both DATA:{n,m} and DATA:*.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/pattern-reference.xlsx
+++ b/docs/pattern-reference.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F94"/>
+  <dimension ref="A1:F96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1273,90 +1273,86 @@
       <c r="D46" s="1" t="inlineStr"/>
       <c r="E46" s="1" t="inlineStr">
         <is>
+          <t>seek:G5    repositions the cursor to G5 WITHOUT reading it. Next cell:next starts from there.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="1" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B47" s="1" t="inlineStr"/>
+      <c r="C47" s="1" t="inlineStr"/>
+      <c r="D47" s="1" t="inlineStr"/>
+      <c r="E47" s="1" t="inlineStr">
+        <is>
           <t>table:*    finds all instances of a repeating table block.</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="6" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="6" t="inlineStr">
         <is>
           <t>START:</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="7" t="inlineStr">
-        <is>
-          <t>cell:A1</t>
-        </is>
-      </c>
-      <c r="B48" s="7" t="inlineStr">
-        <is>
-          <t>po_label</t>
-        </is>
-      </c>
-      <c r="C48" s="7" t="inlineStr"/>
-      <c r="D48" s="7" t="inlineStr"/>
-      <c r="E48" s="7" t="inlineStr">
-        <is>
-          <t>Jump to A1 and read "PO Number:" anchor (lbl: field — not in output).</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
         <is>
-          <t>cell:next</t>
+          <t>cell:A1</t>
         </is>
       </c>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>po.number</t>
+          <t>po_label</t>
         </is>
       </c>
       <c r="C49" s="7" t="inlineStr"/>
       <c r="D49" s="7" t="inlineStr"/>
       <c r="E49" s="7" t="inlineStr">
         <is>
-          <t>Read next non-empty cell after A1 → the PO number.</t>
+          <t>Jump to A1 and read "PO Number:" anchor (lbl: field — not in output).</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
         <is>
-          <t>cell:C1</t>
+          <t>cell:next</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>date_label</t>
+          <t>po.number</t>
         </is>
       </c>
       <c r="C50" s="7" t="inlineStr"/>
       <c r="D50" s="7" t="inlineStr"/>
       <c r="E50" s="7" t="inlineStr">
         <is>
-          <t>Jump to C1 and read "Date:" anchor.</t>
+          <t>Read next non-empty cell after A1 → the PO number.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
         <is>
-          <t>cell:next</t>
+          <t>cell:C1</t>
         </is>
       </c>
       <c r="B51" s="7" t="inlineStr">
         <is>
-          <t>po.date</t>
+          <t>date_label</t>
         </is>
       </c>
       <c r="C51" s="7" t="inlineStr"/>
       <c r="D51" s="7" t="inlineStr"/>
       <c r="E51" s="7" t="inlineStr">
         <is>
-          <t>Read next non-empty cell after C1 → the PO date.</t>
+          <t>Jump to C1 and read "Date:" anchor.</t>
         </is>
       </c>
     </row>
@@ -1368,14 +1364,14 @@
       </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>vendor_label</t>
+          <t>po.date</t>
         </is>
       </c>
       <c r="C52" s="7" t="inlineStr"/>
       <c r="D52" s="7" t="inlineStr"/>
       <c r="E52" s="7" t="inlineStr">
         <is>
-          <t>Read next non-empty cell → "Vendor:" anchor.</t>
+          <t>Read next non-empty cell after C1 → the PO date.</t>
         </is>
       </c>
     </row>
@@ -1387,63 +1383,67 @@
       </c>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t>vendor.name</t>
+          <t>vendor_label</t>
         </is>
       </c>
       <c r="C53" s="7" t="inlineStr"/>
       <c r="D53" s="7" t="inlineStr"/>
       <c r="E53" s="7" t="inlineStr">
         <is>
+          <t>Read next non-empty cell → "Vendor:" anchor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="7" t="inlineStr">
+        <is>
+          <t>cell:next</t>
+        </is>
+      </c>
+      <c r="B54" s="7" t="inlineStr">
+        <is>
+          <t>vendor.name</t>
+        </is>
+      </c>
+      <c r="C54" s="7" t="inlineStr"/>
+      <c r="D54" s="7" t="inlineStr"/>
+      <c r="E54" s="7" t="inlineStr">
+        <is>
           <t>Extract the vendor name.</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="1" t="inlineStr">
-        <is>
-          <t>doc:</t>
-        </is>
-      </c>
-      <c r="B54" s="1" t="inlineStr"/>
-      <c r="C54" s="1" t="inlineStr"/>
-      <c r="D54" s="1" t="inlineStr"/>
-      <c r="E54" s="1" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="1" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B55" s="1" t="inlineStr"/>
+      <c r="C55" s="1" t="inlineStr"/>
+      <c r="D55" s="1" t="inlineStr"/>
+      <c r="E55" s="1" t="inlineStr">
         <is>
           <t>Use IGNORE to skip a non-empty cell without defining a field for it.</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="7" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="7" t="inlineStr">
         <is>
           <t>cell:next</t>
         </is>
       </c>
-      <c r="B55" s="7" t="inlineStr">
+      <c r="B56" s="7" t="inlineStr">
         <is>
           <t>IGNORE</t>
         </is>
       </c>
-      <c r="C55" s="7" t="inlineStr"/>
-      <c r="D55" s="7" t="inlineStr"/>
-      <c r="E55" s="7" t="inlineStr">
+      <c r="C56" s="7" t="inlineStr"/>
+      <c r="D56" s="7" t="inlineStr"/>
+      <c r="E56" s="7" t="inlineStr">
         <is>
           <t>Skip one non-empty cell without capturing it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="1" t="inlineStr">
-        <is>
-          <t>doc:</t>
-        </is>
-      </c>
-      <c r="B57" s="1" t="inlineStr"/>
-      <c r="C57" s="1" t="inlineStr"/>
-      <c r="D57" s="1" t="inlineStr"/>
-      <c r="E57" s="1" t="inlineStr">
-        <is>
-          <t>table:* matches 0-or-more mini-table instances in greedy order.</t>
         </is>
       </c>
     </row>
@@ -1458,42 +1458,29 @@
       <c r="D58" s="1" t="inlineStr"/>
       <c r="E58" s="1" t="inlineStr">
         <is>
+          <t>table:* matches 0-or-more mini-table instances in greedy order.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="1" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B59" s="1" t="inlineStr"/>
+      <c r="C59" s="1" t="inlineStr"/>
+      <c r="D59" s="1" t="inlineStr"/>
+      <c r="E59" s="1" t="inlineStr">
+        <is>
           <t>Use table:1 when exactly one instance is expected.</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="7" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="7" t="inlineStr">
         <is>
           <t>table:*</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="8" t="n"/>
-      <c r="B60" s="8" t="inlineStr">
-        <is>
-          <t>HEADER:1</t>
-        </is>
-      </c>
-      <c r="C60" s="8" t="inlineStr">
-        <is>
-          <t>col_item</t>
-        </is>
-      </c>
-      <c r="D60" s="8" t="inlineStr">
-        <is>
-          <t>col_qty</t>
-        </is>
-      </c>
-      <c r="E60" s="8" t="inlineStr">
-        <is>
-          <t>col_price</t>
-        </is>
-      </c>
-      <c r="F60" s="8" t="inlineStr">
-        <is>
-          <t>col_total</t>
         </is>
       </c>
     </row>
@@ -1501,27 +1488,27 @@
       <c r="A61" s="8" t="n"/>
       <c r="B61" s="8" t="inlineStr">
         <is>
-          <t>DATA:*</t>
+          <t>HEADER:1</t>
         </is>
       </c>
       <c r="C61" s="8" t="inlineStr">
         <is>
-          <t>line.item</t>
+          <t>col_item</t>
         </is>
       </c>
       <c r="D61" s="8" t="inlineStr">
         <is>
-          <t>line.qty</t>
+          <t>col_qty</t>
         </is>
       </c>
       <c r="E61" s="8" t="inlineStr">
         <is>
-          <t>line.price</t>
+          <t>col_price</t>
         </is>
       </c>
       <c r="F61" s="8" t="inlineStr">
         <is>
-          <t>line.total</t>
+          <t>col_total</t>
         </is>
       </c>
     </row>
@@ -1529,42 +1516,55 @@
       <c r="A62" s="8" t="n"/>
       <c r="B62" s="8" t="inlineStr">
         <is>
+          <t>DATA:*</t>
+        </is>
+      </c>
+      <c r="C62" s="8" t="inlineStr">
+        <is>
+          <t>line.item</t>
+        </is>
+      </c>
+      <c r="D62" s="8" t="inlineStr">
+        <is>
+          <t>line.qty</t>
+        </is>
+      </c>
+      <c r="E62" s="8" t="inlineStr">
+        <is>
+          <t>line.price</t>
+        </is>
+      </c>
+      <c r="F62" s="8" t="inlineStr">
+        <is>
+          <t>line.total</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="8" t="n"/>
+      <c r="B63" s="8" t="inlineStr">
+        <is>
           <t>FOOTER:1</t>
         </is>
       </c>
-      <c r="C62" s="8" t="inlineStr">
+      <c r="C63" s="8" t="inlineStr">
         <is>
           <t>footer.label</t>
         </is>
       </c>
-      <c r="D62" s="8" t="inlineStr">
+      <c r="D63" s="8" t="inlineStr">
         <is>
           <t>IGNORE</t>
         </is>
       </c>
-      <c r="E62" s="8" t="inlineStr">
+      <c r="E63" s="8" t="inlineStr">
         <is>
           <t>IGNORE</t>
         </is>
       </c>
-      <c r="F62" s="8" t="inlineStr">
+      <c r="F63" s="8" t="inlineStr">
         <is>
           <t>footer.value</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="1" t="inlineStr">
-        <is>
-          <t>doc:</t>
-        </is>
-      </c>
-      <c r="B63" s="1" t="inlineStr"/>
-      <c r="C63" s="1" t="inlineStr"/>
-      <c r="D63" s="1" t="inlineStr"/>
-      <c r="E63" s="1" t="inlineStr">
-        <is>
-          <t>HEADER/FOOTER are strict: wrong or missing value = no match.</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="D64" s="1" t="inlineStr"/>
       <c r="E64" s="1" t="inlineStr">
         <is>
-          <t>DATA rows are lenient: wrong value emits a warning but extraction continues.</t>
+          <t>HEADER/FOOTER are strict: wrong or missing value = no match.</t>
         </is>
       </c>
     </row>
@@ -1594,7 +1594,7 @@
       <c r="D65" s="1" t="inlineStr"/>
       <c r="E65" s="1" t="inlineStr">
         <is>
-          <t>EMPTY column keyword: cell must be blank. IGNORE: consume without matching.</t>
+          <t>DATA rows are lenient: wrong value emits a warning but extraction continues.</t>
         </is>
       </c>
     </row>
@@ -1609,7 +1609,7 @@
       <c r="D66" s="1" t="inlineStr"/>
       <c r="E66" s="1" t="inlineStr">
         <is>
-          <t>── BOUNDED DATA + SKIP_IF (fixed-slot templates) ───────────────────────</t>
+          <t>EMPTY column keyword: cell must be blank. IGNORE: consume without matching.</t>
         </is>
       </c>
     </row>
@@ -1624,7 +1624,7 @@
       <c r="D67" s="1" t="inlineStr"/>
       <c r="E67" s="1" t="inlineStr">
         <is>
-          <t>Use DATA:{n,m} when the template pre-allocates a fixed number of rows.</t>
+          <t>── BOUNDED DATA + SKIP_IF (fixed-slot templates) ───────────────────────</t>
         </is>
       </c>
     </row>
@@ -1639,7 +1639,7 @@
       <c r="D68" s="1" t="inlineStr"/>
       <c r="E68" s="1" t="inlineStr">
         <is>
-          <t>n = min total physical rows expected, m = max total rows to scan.</t>
+          <t>Use DATA:{n,m} when the template pre-allocates a fixed number of rows.</t>
         </is>
       </c>
     </row>
@@ -1654,7 +1654,7 @@
       <c r="D69" s="1" t="inlineStr"/>
       <c r="E69" s="1" t="inlineStr">
         <is>
-          <t>SKIP_IF: rows matching the condition are silently excluded from output</t>
+          <t>n = min total physical rows expected, m = max total rows to scan.</t>
         </is>
       </c>
     </row>
@@ -1669,7 +1669,7 @@
       <c r="D70" s="1" t="inlineStr"/>
       <c r="E70" s="1" t="inlineStr">
         <is>
-          <t>but still count toward the {n,m} bounds.</t>
+          <t>SKIP_IF: rows matching the condition are silently excluded from output</t>
         </is>
       </c>
     </row>
@@ -1684,32 +1684,29 @@
       <c r="D71" s="1" t="inlineStr"/>
       <c r="E71" s="1" t="inlineStr">
         <is>
-          <t>SKIP_IF is only valid with DATA:{n,m}.</t>
+          <t>but still count toward the {n,m} bounds.</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="7" t="inlineStr">
+      <c r="A72" s="1" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B72" s="1" t="inlineStr"/>
+      <c r="C72" s="1" t="inlineStr"/>
+      <c r="D72" s="1" t="inlineStr"/>
+      <c r="E72" s="1" t="inlineStr">
+        <is>
+          <t>SKIP_IF is valid with DATA:{n,m} (rows count toward bounds) and DATA:* (rows filtered, scan continues).</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="7" t="inlineStr">
         <is>
           <t>table:1</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="8" t="n"/>
-      <c r="B73" s="8" t="inlineStr">
-        <is>
-          <t>HEADER:1</t>
-        </is>
-      </c>
-      <c r="C73" s="8" t="inlineStr">
-        <is>
-          <t>col_item</t>
-        </is>
-      </c>
-      <c r="D73" s="8" t="inlineStr">
-        <is>
-          <t>col_qty</t>
         </is>
       </c>
     </row>
@@ -1717,17 +1714,17 @@
       <c r="A74" s="8" t="n"/>
       <c r="B74" s="8" t="inlineStr">
         <is>
-          <t>SKIP_IF</t>
+          <t>HEADER:1</t>
         </is>
       </c>
       <c r="C74" s="8" t="inlineStr">
         <is>
-          <t>EMPTY</t>
+          <t>col_item</t>
         </is>
       </c>
       <c r="D74" s="8" t="inlineStr">
         <is>
-          <t>IGNORE</t>
+          <t>col_qty</t>
         </is>
       </c>
     </row>
@@ -1735,17 +1732,17 @@
       <c r="A75" s="8" t="n"/>
       <c r="B75" s="8" t="inlineStr">
         <is>
-          <t>DATA:{0,15}</t>
+          <t>SKIP_IF</t>
         </is>
       </c>
       <c r="C75" s="8" t="inlineStr">
         <is>
-          <t>line.item</t>
+          <t>EMPTY</t>
         </is>
       </c>
       <c r="D75" s="8" t="inlineStr">
         <is>
-          <t>line.qty</t>
+          <t>IGNORE</t>
         </is>
       </c>
     </row>
@@ -1753,39 +1750,42 @@
       <c r="A76" s="8" t="n"/>
       <c r="B76" s="8" t="inlineStr">
         <is>
+          <t>DATA:{0,15}</t>
+        </is>
+      </c>
+      <c r="C76" s="8" t="inlineStr">
+        <is>
+          <t>line.item</t>
+        </is>
+      </c>
+      <c r="D76" s="8" t="inlineStr">
+        <is>
+          <t>line.qty</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="8" t="n"/>
+      <c r="B77" s="8" t="inlineStr">
+        <is>
           <t>FOOTER:1</t>
         </is>
       </c>
-      <c r="C76" s="8" t="inlineStr">
+      <c r="C77" s="8" t="inlineStr">
         <is>
           <t>lbl_total</t>
         </is>
       </c>
-      <c r="D76" s="8" t="inlineStr">
+      <c r="D77" s="8" t="inlineStr">
         <is>
           <t>inv.total</t>
         </is>
       </c>
     </row>
-    <row r="78">
-      <c r="A78" s="6" t="inlineStr">
+    <row r="79">
+      <c r="A79" s="6" t="inlineStr">
         <is>
           <t>END:</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="1" t="inlineStr">
-        <is>
-          <t>doc:</t>
-        </is>
-      </c>
-      <c r="B80" s="1" t="inlineStr"/>
-      <c r="C80" s="1" t="inlineStr"/>
-      <c r="D80" s="1" t="inlineStr"/>
-      <c r="E80" s="1" t="inlineStr">
-        <is>
-          <t>── QUICK REFERENCE ──────────────────────────────────────────────</t>
         </is>
       </c>
     </row>
@@ -1795,87 +1795,84 @@
           <t>doc:</t>
         </is>
       </c>
-      <c r="B81" s="1" t="inlineStr">
+      <c r="B81" s="1" t="inlineStr"/>
+      <c r="C81" s="1" t="inlineStr"/>
+      <c r="D81" s="1" t="inlineStr"/>
+      <c r="E81" s="1" t="inlineStr">
+        <is>
+          <t>── QUICK REFERENCE ──────────────────────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="1" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B82" s="1" t="inlineStr">
         <is>
           <t>doc: | free text</t>
         </is>
       </c>
-      <c r="C81" s="1" t="inlineStr"/>
-      <c r="D81" s="1" t="inlineStr">
+      <c r="C82" s="1" t="inlineStr"/>
+      <c r="D82" s="1" t="inlineStr">
         <is>
           <t>Inline comment. Ignored by engine.</t>
         </is>
       </c>
     </row>
-    <row r="82">
-      <c r="A82" s="3" t="inlineStr">
+    <row r="83">
+      <c r="A83" s="3" t="inlineStr">
         <is>
           <t>config:</t>
         </is>
       </c>
-      <c r="B82" s="3" t="inlineStr">
+      <c r="B83" s="3" t="inlineStr">
         <is>
           <t>config: | key | value</t>
         </is>
       </c>
-      <c r="C82" s="3" t="inlineStr"/>
-      <c r="D82" s="3" t="inlineStr">
+      <c r="C83" s="3" t="inlineStr"/>
+      <c r="D83" s="3" t="inlineStr">
         <is>
           <t>Global setting. Keys: read.direction, currency.sign, empty.aliases, ignore.case</t>
         </is>
       </c>
     </row>
-    <row r="83">
-      <c r="A83" s="4" t="inlineStr">
+    <row r="84">
+      <c r="A84" s="4" t="inlineStr">
         <is>
           <t>lbl:</t>
         </is>
       </c>
-      <c r="B83" s="4" t="inlineStr">
+      <c r="B84" s="4" t="inlineStr">
         <is>
           <t>lbl: | name | type | regex</t>
         </is>
       </c>
-      <c r="C83" s="4" t="inlineStr"/>
-      <c r="D83" s="4" t="inlineStr">
+      <c r="C84" s="4" t="inlineStr"/>
+      <c r="D84" s="4" t="inlineStr">
         <is>
           <t>Anchor label. Matched but never in output.</t>
         </is>
       </c>
     </row>
-    <row r="84">
-      <c r="A84" s="5" t="inlineStr">
+    <row r="85">
+      <c r="A85" s="5" t="inlineStr">
         <is>
           <t>var:</t>
         </is>
       </c>
-      <c r="B84" s="5" t="inlineStr">
+      <c r="B85" s="5" t="inlineStr">
         <is>
           <t>var: | name | type | regex</t>
         </is>
       </c>
-      <c r="C84" s="5" t="inlineStr"/>
-      <c r="D84" s="5" t="inlineStr">
+      <c r="C85" s="5" t="inlineStr"/>
+      <c r="D85" s="5" t="inlineStr">
         <is>
           <t>Extracted variable. Use dot notation for nesting.</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" t="inlineStr">
-        <is>
-          <t>cell:next</t>
-        </is>
-      </c>
-      <c r="B85" t="inlineStr">
-        <is>
-          <t>cell:next | FieldName</t>
-        </is>
-      </c>
-      <c r="C85" t="inlineStr"/>
-      <c r="D85" t="inlineStr">
-        <is>
-          <t>Read next non-empty cell (alias: cell:1).</t>
         </is>
       </c>
     </row>
@@ -1887,13 +1884,13 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>cell:next | IGNORE</t>
+          <t>cell:next | FieldName</t>
         </is>
       </c>
       <c r="C86" t="inlineStr"/>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Skip next non-empty cell without capturing.</t>
+          <t>Read next non-empty cell (alias: cell:1).</t>
         </is>
       </c>
     </row>
@@ -1905,137 +1902,173 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>cell:B5 | FieldName</t>
+          <t>cell:next | IGNORE</t>
         </is>
       </c>
       <c r="C87" t="inlineStr"/>
       <c r="D87" t="inlineStr">
         <is>
+          <t>Skip next non-empty cell without capturing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>cell:next</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>cell:B5 | FieldName</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr"/>
+      <c r="D88" t="inlineStr">
+        <is>
           <t>Jump directly to B5 (absolute reference). Ordering must be forward.</t>
         </is>
       </c>
     </row>
-    <row r="88">
-      <c r="A88" s="7" t="inlineStr">
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>seek:</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>seek:G5</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr"/>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Reposition cursor to G5 without reading it. Resets abs-ref ordering constraint.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="7" t="inlineStr">
         <is>
           <t>table:*</t>
         </is>
       </c>
-      <c r="B88" s="7" t="inlineStr">
+      <c r="B90" s="7" t="inlineStr">
         <is>
           <t>table:*  (or table:1)</t>
         </is>
       </c>
-      <c r="C88" s="7" t="inlineStr"/>
-      <c r="D88" s="7" t="inlineStr">
+      <c r="C90" s="7" t="inlineStr"/>
+      <c r="D90" s="7" t="inlineStr">
         <is>
           <t>Begin a repeating table block.</t>
-        </is>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" s="8" t="inlineStr">
-        <is>
-          <t>HEADER:N</t>
-        </is>
-      </c>
-      <c r="B89" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> | HEADER:1 | F1 | F2</t>
-        </is>
-      </c>
-      <c r="C89" s="8" t="inlineStr"/>
-      <c r="D89" s="8" t="inlineStr">
-        <is>
-          <t>Strict header row template (col A must be blank).</t>
-        </is>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" s="8" t="inlineStr">
-        <is>
-          <t>DATA:*</t>
-        </is>
-      </c>
-      <c r="B90" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> | DATA:* | F1 | F2</t>
-        </is>
-      </c>
-      <c r="C90" s="8" t="inlineStr"/>
-      <c r="D90" s="8" t="inlineStr">
-        <is>
-          <t>Data row template (greedy, lenient validation).</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="8" t="inlineStr">
         <is>
-          <t>DATA:{n,m}</t>
+          <t>HEADER:N</t>
         </is>
       </c>
       <c r="B91" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | DATA:{0,15} | F1 | F2</t>
+          <t xml:space="preserve"> | HEADER:1 | F1 | F2</t>
         </is>
       </c>
       <c r="C91" s="8" t="inlineStr"/>
       <c r="D91" s="8" t="inlineStr">
         <is>
-          <t>Bounded data: scan at most m physical rows, warn if &lt; n.</t>
+          <t>Strict header row template (col A must be blank).</t>
         </is>
       </c>
     </row>
     <row r="92">
-      <c r="A92" t="inlineStr">
-        <is>
-          <t>SKIP_IF</t>
-        </is>
-      </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> | SKIP_IF | EMPTY | IGNORE</t>
-        </is>
-      </c>
-      <c r="C92" t="inlineStr"/>
-      <c r="D92" t="inlineStr">
-        <is>
-          <t>Skip row if non-IGNORE columns match. Only with DATA:{n,m}.</t>
+      <c r="A92" s="8" t="inlineStr">
+        <is>
+          <t>DATA:*</t>
+        </is>
+      </c>
+      <c r="B92" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> | DATA:* | F1 | F2</t>
+        </is>
+      </c>
+      <c r="C92" s="8" t="inlineStr"/>
+      <c r="D92" s="8" t="inlineStr">
+        <is>
+          <t>Data row template (greedy, lenient validation).</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="8" t="inlineStr">
         <is>
-          <t>FOOTER:N</t>
+          <t>DATA:{n,m}</t>
         </is>
       </c>
       <c r="B93" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | FOOTER:1 | F1 | F2</t>
+          <t xml:space="preserve"> | DATA:{0,15} | F1 | F2</t>
         </is>
       </c>
       <c r="C93" s="8" t="inlineStr"/>
       <c r="D93" s="8" t="inlineStr">
         <is>
+          <t>Bounded data: scan at most m physical rows, warn if &lt; n.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>SKIP_IF</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> | SKIP_IF | EMPTY | IGNORE</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr"/>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Skip row if non-IGNORE columns match. Valid with DATA:{n,m} and DATA:*.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="8" t="inlineStr">
+        <is>
+          <t>FOOTER:N</t>
+        </is>
+      </c>
+      <c r="B95" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> | FOOTER:1 | F1 | F2</t>
+        </is>
+      </c>
+      <c r="C95" s="8" t="inlineStr"/>
+      <c r="D95" s="8" t="inlineStr">
+        <is>
           <t>Strict footer row template.</t>
         </is>
       </c>
     </row>
-    <row r="94">
-      <c r="A94" s="8" t="inlineStr">
+    <row r="96">
+      <c r="A96" s="8" t="inlineStr">
         <is>
           <t>SPLITTER</t>
         </is>
       </c>
-      <c r="B94" s="8" t="inlineStr">
+      <c r="B96" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve"> | SPLITTER:1</t>
         </is>
       </c>
-      <c r="C94" s="8" t="inlineStr"/>
-      <c r="D94" s="8" t="inlineStr">
+      <c r="C96" s="8" t="inlineStr"/>
+      <c r="D96" s="8" t="inlineStr">
         <is>
           <t>All columns must be blank (separator row).</t>
         </is>

</xml_diff>

<commit_message>
feat(pattern): stamp pattern.version:1 into generated patterns
draft (PatternWriter) and the docs reference now emit an explicit
config: | pattern.version | 1 so machine-generated patterns are version-explicit
by default (skipped if the model already emitted one). Reference regenerated.

Completes #29. Full suite 1178 passed.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/pattern-reference.xlsx
+++ b/docs/pattern-reference.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F97"/>
+  <dimension ref="A1:F98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -578,18 +578,18 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>read.direction</t>
+          <t>pattern.version</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>LR</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr"/>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>LR = left-to-right scan (default). TD = top-to-bottom.</t>
+          <t>Pattern-format version (optional; absent = 1). Engine errors if newer than it understands.</t>
         </is>
       </c>
     </row>
@@ -601,18 +601,18 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>currency.sign</t>
+          <t>read.direction</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>€</t>
+          <t>LR</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr"/>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>Symbol used when parsing currency values.</t>
+          <t>LR = left-to-right scan (default). TD = top-to-bottom.</t>
         </is>
       </c>
     </row>
@@ -624,33 +624,41 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>ignore.case</t>
+          <t>currency.sign</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>€</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr"/>
       <c r="E13" s="3" t="inlineStr">
         <is>
+          <t>Symbol used when parsing currency values.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>config:</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>ignore.case</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr"/>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
           <t>yes = match all regexes case-insensitively. Default no.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>doc:</t>
-        </is>
-      </c>
-      <c r="B15" s="1" t="inlineStr"/>
-      <c r="C15" s="1" t="inlineStr"/>
-      <c r="D15" s="1" t="inlineStr"/>
-      <c r="E15" s="1" t="inlineStr">
-        <is>
-          <t>lbl: defines an anchor label. Matched for position only — NEVER written to output JSON.</t>
         </is>
       </c>
     </row>
@@ -665,34 +673,22 @@
       <c r="D16" s="1" t="inlineStr"/>
       <c r="E16" s="1" t="inlineStr">
         <is>
+          <t>lbl: defines an anchor label. Matched for position only — NEVER written to output JSON.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="inlineStr"/>
+      <c r="C17" s="1" t="inlineStr"/>
+      <c r="D17" s="1" t="inlineStr"/>
+      <c r="E17" s="1" t="inlineStr">
+        <is>
           <t>Use lbl: for literal text like "Invoice No:" or table column headers like "Product".</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>lbl:</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>po_label</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>PO Number:</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>Matches the literal text "PO Number:" in the sheet.</t>
         </is>
       </c>
     </row>
@@ -704,7 +700,7 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>date_label</t>
+          <t>po_label</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
@@ -714,12 +710,12 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Date:</t>
+          <t>PO Number:</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>Matches "Date:".</t>
+          <t>Matches the literal text "PO Number:" in the sheet.</t>
         </is>
       </c>
     </row>
@@ -731,7 +727,7 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>vendor_label</t>
+          <t>date_label</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
@@ -741,12 +737,12 @@
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Vendor:</t>
+          <t>Date:</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>Matches "Vendor:".</t>
+          <t>Matches "Date:".</t>
         </is>
       </c>
     </row>
@@ -758,7 +754,7 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>col_item</t>
+          <t>vendor_label</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
@@ -768,12 +764,12 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Item</t>
+          <t>Vendor:</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>Table column header anchor.</t>
+          <t>Matches "Vendor:".</t>
         </is>
       </c>
     </row>
@@ -785,7 +781,7 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>col_qty</t>
+          <t>col_item</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
@@ -795,7 +791,7 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Qty</t>
+          <t>Item</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
@@ -812,7 +808,7 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>col_price</t>
+          <t>col_qty</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
@@ -822,7 +818,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Unit Price</t>
+          <t>Qty</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
@@ -839,37 +835,49 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
+          <t>col_price</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Unit Price</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>Table column header anchor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>lbl:</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
           <t>col_total</t>
         </is>
       </c>
-      <c r="C23" s="4" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
+      <c r="D24" s="4" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="E23" s="4" t="inlineStr">
+      <c r="E24" s="4" t="inlineStr">
         <is>
           <t>Table column header anchor.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="1" t="inlineStr">
-        <is>
-          <t>doc:</t>
-        </is>
-      </c>
-      <c r="B25" s="1" t="inlineStr"/>
-      <c r="C25" s="1" t="inlineStr"/>
-      <c r="D25" s="1" t="inlineStr"/>
-      <c r="E25" s="1" t="inlineStr">
-        <is>
-          <t>var: defines a data field. Extracted and written to output JSON.</t>
         </is>
       </c>
     </row>
@@ -884,7 +892,7 @@
       <c r="D26" s="1" t="inlineStr"/>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>Dot notation creates nested JSON: po.number → {"po": {"number": ...}}</t>
+          <t>var: defines a data field. Extracted and written to output JSON.</t>
         </is>
       </c>
     </row>
@@ -899,7 +907,7 @@
       <c r="D27" s="1" t="inlineStr"/>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>All var: fields in one table DATA row must share the same group prefix.</t>
+          <t>Dot notation creates nested JSON: po.number → {"po": {"number": ...}}</t>
         </is>
       </c>
     </row>
@@ -914,7 +922,7 @@
       <c r="D28" s="1" t="inlineStr"/>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>Types: string text integer number/float/decimal currency percentage boolean time duration date datetime</t>
+          <t>All var: fields in one table DATA row must share the same group prefix.</t>
         </is>
       </c>
     </row>
@@ -929,7 +937,7 @@
       <c r="D29" s="1" t="inlineStr"/>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>Regex: Python re.fullmatch pattern. Leave blank (or .*) to accept any value of the declared type.</t>
+          <t>Types: string text integer number/float/decimal currency percentage boolean time duration date datetime</t>
         </is>
       </c>
     </row>
@@ -944,7 +952,7 @@
       <c r="D30" s="1" t="inlineStr"/>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>Comments: a doc:/info: row is a whole-line comment. On config/var/lbl/cell/START rows,</t>
+          <t>Regex: Python re.fullmatch pattern. Leave blank (or .*) to accept any value of the declared type.</t>
         </is>
       </c>
     </row>
@@ -959,7 +967,7 @@
       <c r="D31" s="1" t="inlineStr"/>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>a cell starting with # AFTER the real columns is a trailing comment to end of row</t>
+          <t>Comments: a doc:/info: row is a whole-line comment. On config/var/lbl/cell/START rows,</t>
         </is>
       </c>
     </row>
@@ -974,34 +982,22 @@
       <c r="D32" s="1" t="inlineStr"/>
       <c r="E32" s="1" t="inlineStr">
         <is>
+          <t>a cell starting with # AFTER the real columns is a trailing comment to end of row</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B33" s="1" t="inlineStr"/>
+      <c r="C33" s="1" t="inlineStr"/>
+      <c r="D33" s="1" t="inlineStr"/>
+      <c r="E33" s="1" t="inlineStr">
+        <is>
           <t>(var:/lbl: → col E+, cell: → col C+, config: → col D+). NOT in table: rows (# is literal there).</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="5" t="inlineStr">
-        <is>
-          <t>var:</t>
-        </is>
-      </c>
-      <c r="B33" s="5" t="inlineStr">
-        <is>
-          <t>po.number</t>
-        </is>
-      </c>
-      <c r="C33" s="5" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="D33" s="5" t="inlineStr">
-        <is>
-          <t>PO-[0-9]{4}</t>
-        </is>
-      </c>
-      <c r="E33" s="5" t="inlineStr">
-        <is>
-          <t>Matches e.g. "PO-2026". Output key: {"po": {"number": ...}}</t>
         </is>
       </c>
     </row>
@@ -1013,18 +1009,22 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>po.date</t>
+          <t>po.number</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>date</t>
-        </is>
-      </c>
-      <c r="D34" s="5" t="inlineStr"/>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>PO-[0-9]{4}</t>
+        </is>
+      </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>Any date value. Regex left empty → defaults to .*</t>
+          <t>Matches e.g. "PO-2026". Output key: {"po": {"number": ...}}</t>
         </is>
       </c>
     </row>
@@ -1036,22 +1036,18 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>vendor.name</t>
+          <t>po.date</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="D35" s="5" t="inlineStr">
-        <is>
-          <t>.+</t>
-        </is>
-      </c>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr"/>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>Any non-empty string.</t>
+          <t>Any date value. Regex left empty → defaults to .*</t>
         </is>
       </c>
     </row>
@@ -1063,7 +1059,7 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>line.item</t>
+          <t>vendor.name</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
@@ -1078,7 +1074,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>Table DATA field. Group prefix "line" → {"line": [...]}</t>
+          <t>Any non-empty string.</t>
         </is>
       </c>
     </row>
@@ -1090,22 +1086,22 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>line.qty</t>
+          <t>line.item</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>string</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>[1-9][0-9]*</t>
+          <t>.+</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>Positive integer.</t>
+          <t>Table DATA field. Group prefix "line" → {"line": [...]}</t>
         </is>
       </c>
     </row>
@@ -1117,22 +1113,22 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>line.price</t>
+          <t>line.qty</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>currency</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>.*</t>
+          <t>[1-9][0-9]*</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>Any currency value.</t>
+          <t>Positive integer.</t>
         </is>
       </c>
     </row>
@@ -1144,7 +1140,7 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>line.total</t>
+          <t>line.price</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
@@ -1171,22 +1167,22 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>footer.label</t>
+          <t>line.total</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>currency</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>Grand Total</t>
+          <t>.*</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t>FOOTER field — matches the literal "Grand Total".</t>
+          <t>Any currency value.</t>
         </is>
       </c>
     </row>
@@ -1198,37 +1194,49 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
+          <t>footer.label</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>Grand Total</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>FOOTER field — matches the literal "Grand Total".</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>var:</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
           <t>footer.value</t>
         </is>
       </c>
-      <c r="C41" s="5" t="inlineStr">
+      <c r="C42" s="5" t="inlineStr">
         <is>
           <t>currency</t>
         </is>
       </c>
-      <c r="D41" s="5" t="inlineStr">
+      <c r="D42" s="5" t="inlineStr">
         <is>
           <t>.*</t>
         </is>
       </c>
-      <c r="E41" s="5" t="inlineStr">
+      <c r="E42" s="5" t="inlineStr">
         <is>
           <t>FOOTER value field.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="1" t="inlineStr">
-        <is>
-          <t>doc:</t>
-        </is>
-      </c>
-      <c r="B43" s="1" t="inlineStr"/>
-      <c r="C43" s="1" t="inlineStr"/>
-      <c r="D43" s="1" t="inlineStr"/>
-      <c r="E43" s="1" t="inlineStr">
-        <is>
-          <t>Everything between START: and END: defines the extraction order.</t>
         </is>
       </c>
     </row>
@@ -1243,7 +1251,7 @@
       <c r="D44" s="1" t="inlineStr"/>
       <c r="E44" s="1" t="inlineStr">
         <is>
-          <t>cell:next  reads the next non-empty cell (alias: cell:1). Scans in read.direction order.</t>
+          <t>Everything between START: and END: defines the extraction order.</t>
         </is>
       </c>
     </row>
@@ -1258,7 +1266,7 @@
       <c r="D45" s="1" t="inlineStr"/>
       <c r="E45" s="1" t="inlineStr">
         <is>
-          <t>cell:B5    jumps directly to cell B5 (absolute A1-notation reference).</t>
+          <t>cell:next  reads the next non-empty cell (alias: cell:1). Scans in read.direction order.</t>
         </is>
       </c>
     </row>
@@ -1273,7 +1281,7 @@
       <c r="D46" s="1" t="inlineStr"/>
       <c r="E46" s="1" t="inlineStr">
         <is>
-          <t>seek:G5    repositions the cursor to G5 WITHOUT reading it. Next cell:next starts from there.</t>
+          <t>cell:B5    jumps directly to cell B5 (absolute A1-notation reference).</t>
         </is>
       </c>
     </row>
@@ -1288,7 +1296,7 @@
       <c r="D47" s="1" t="inlineStr"/>
       <c r="E47" s="1" t="inlineStr">
         <is>
-          <t>dir:LR     switches scan direction to left-to-right from here on (dir:TD = top-down).</t>
+          <t>seek:G5    repositions the cursor to G5 WITHOUT reading it. Next cell:next starts from there.</t>
         </is>
       </c>
     </row>
@@ -1303,90 +1311,86 @@
       <c r="D48" s="1" t="inlineStr"/>
       <c r="E48" s="1" t="inlineStr">
         <is>
+          <t>dir:LR     switches scan direction to left-to-right from here on (dir:TD = top-down).</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="1" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B49" s="1" t="inlineStr"/>
+      <c r="C49" s="1" t="inlineStr"/>
+      <c r="D49" s="1" t="inlineStr"/>
+      <c r="E49" s="1" t="inlineStr">
+        <is>
           <t>table:*    finds all instances of a repeating table block.</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="6" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="6" t="inlineStr">
         <is>
           <t>START:</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="7" t="inlineStr">
-        <is>
-          <t>cell:A1</t>
-        </is>
-      </c>
-      <c r="B50" s="7" t="inlineStr">
-        <is>
-          <t>po_label</t>
-        </is>
-      </c>
-      <c r="C50" s="7" t="inlineStr"/>
-      <c r="D50" s="7" t="inlineStr"/>
-      <c r="E50" s="7" t="inlineStr">
-        <is>
-          <t>Jump to A1 and read "PO Number:" anchor (lbl: field — not in output).</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
         <is>
-          <t>cell:next</t>
+          <t>cell:A1</t>
         </is>
       </c>
       <c r="B51" s="7" t="inlineStr">
         <is>
-          <t>po.number</t>
+          <t>po_label</t>
         </is>
       </c>
       <c r="C51" s="7" t="inlineStr"/>
       <c r="D51" s="7" t="inlineStr"/>
       <c r="E51" s="7" t="inlineStr">
         <is>
-          <t>Read next non-empty cell after A1 → the PO number.</t>
+          <t>Jump to A1 and read "PO Number:" anchor (lbl: field — not in output).</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
         <is>
-          <t>cell:C1</t>
+          <t>cell:next</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>date_label</t>
+          <t>po.number</t>
         </is>
       </c>
       <c r="C52" s="7" t="inlineStr"/>
       <c r="D52" s="7" t="inlineStr"/>
       <c r="E52" s="7" t="inlineStr">
         <is>
-          <t>Jump to C1 and read "Date:" anchor.</t>
+          <t>Read next non-empty cell after A1 → the PO number.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
         <is>
-          <t>cell:next</t>
+          <t>cell:C1</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t>po.date</t>
+          <t>date_label</t>
         </is>
       </c>
       <c r="C53" s="7" t="inlineStr"/>
       <c r="D53" s="7" t="inlineStr"/>
       <c r="E53" s="7" t="inlineStr">
         <is>
-          <t>Read next non-empty cell after C1 → the PO date.</t>
+          <t>Jump to C1 and read "Date:" anchor.</t>
         </is>
       </c>
     </row>
@@ -1398,14 +1402,14 @@
       </c>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>vendor_label</t>
+          <t>po.date</t>
         </is>
       </c>
       <c r="C54" s="7" t="inlineStr"/>
       <c r="D54" s="7" t="inlineStr"/>
       <c r="E54" s="7" t="inlineStr">
         <is>
-          <t>Read next non-empty cell → "Vendor:" anchor.</t>
+          <t>Read next non-empty cell after C1 → the PO date.</t>
         </is>
       </c>
     </row>
@@ -1417,63 +1421,67 @@
       </c>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>vendor.name</t>
+          <t>vendor_label</t>
         </is>
       </c>
       <c r="C55" s="7" t="inlineStr"/>
       <c r="D55" s="7" t="inlineStr"/>
       <c r="E55" s="7" t="inlineStr">
         <is>
+          <t>Read next non-empty cell → "Vendor:" anchor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="7" t="inlineStr">
+        <is>
+          <t>cell:next</t>
+        </is>
+      </c>
+      <c r="B56" s="7" t="inlineStr">
+        <is>
+          <t>vendor.name</t>
+        </is>
+      </c>
+      <c r="C56" s="7" t="inlineStr"/>
+      <c r="D56" s="7" t="inlineStr"/>
+      <c r="E56" s="7" t="inlineStr">
+        <is>
           <t>Extract the vendor name.</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="1" t="inlineStr">
-        <is>
-          <t>doc:</t>
-        </is>
-      </c>
-      <c r="B56" s="1" t="inlineStr"/>
-      <c r="C56" s="1" t="inlineStr"/>
-      <c r="D56" s="1" t="inlineStr"/>
-      <c r="E56" s="1" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="1" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B57" s="1" t="inlineStr"/>
+      <c r="C57" s="1" t="inlineStr"/>
+      <c r="D57" s="1" t="inlineStr"/>
+      <c r="E57" s="1" t="inlineStr">
         <is>
           <t>Use IGNORE to skip a non-empty cell without defining a field for it.</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="7" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="7" t="inlineStr">
         <is>
           <t>cell:next</t>
         </is>
       </c>
-      <c r="B57" s="7" t="inlineStr">
+      <c r="B58" s="7" t="inlineStr">
         <is>
           <t>IGNORE</t>
         </is>
       </c>
-      <c r="C57" s="7" t="inlineStr"/>
-      <c r="D57" s="7" t="inlineStr"/>
-      <c r="E57" s="7" t="inlineStr">
+      <c r="C58" s="7" t="inlineStr"/>
+      <c r="D58" s="7" t="inlineStr"/>
+      <c r="E58" s="7" t="inlineStr">
         <is>
           <t>Skip one non-empty cell without capturing it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="1" t="inlineStr">
-        <is>
-          <t>doc:</t>
-        </is>
-      </c>
-      <c r="B59" s="1" t="inlineStr"/>
-      <c r="C59" s="1" t="inlineStr"/>
-      <c r="D59" s="1" t="inlineStr"/>
-      <c r="E59" s="1" t="inlineStr">
-        <is>
-          <t>table:* matches 0-or-more mini-table instances in greedy order.</t>
         </is>
       </c>
     </row>
@@ -1488,42 +1496,29 @@
       <c r="D60" s="1" t="inlineStr"/>
       <c r="E60" s="1" t="inlineStr">
         <is>
+          <t>table:* matches 0-or-more mini-table instances in greedy order.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="1" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B61" s="1" t="inlineStr"/>
+      <c r="C61" s="1" t="inlineStr"/>
+      <c r="D61" s="1" t="inlineStr"/>
+      <c r="E61" s="1" t="inlineStr">
+        <is>
           <t>Use table:1 when exactly one instance is expected.</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="7" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="7" t="inlineStr">
         <is>
           <t>table:*</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="8" t="n"/>
-      <c r="B62" s="8" t="inlineStr">
-        <is>
-          <t>HEADER:1</t>
-        </is>
-      </c>
-      <c r="C62" s="8" t="inlineStr">
-        <is>
-          <t>col_item</t>
-        </is>
-      </c>
-      <c r="D62" s="8" t="inlineStr">
-        <is>
-          <t>col_qty</t>
-        </is>
-      </c>
-      <c r="E62" s="8" t="inlineStr">
-        <is>
-          <t>col_price</t>
-        </is>
-      </c>
-      <c r="F62" s="8" t="inlineStr">
-        <is>
-          <t>col_total</t>
         </is>
       </c>
     </row>
@@ -1531,27 +1526,27 @@
       <c r="A63" s="8" t="n"/>
       <c r="B63" s="8" t="inlineStr">
         <is>
-          <t>DATA:*</t>
+          <t>HEADER:1</t>
         </is>
       </c>
       <c r="C63" s="8" t="inlineStr">
         <is>
-          <t>line.item</t>
+          <t>col_item</t>
         </is>
       </c>
       <c r="D63" s="8" t="inlineStr">
         <is>
-          <t>line.qty</t>
+          <t>col_qty</t>
         </is>
       </c>
       <c r="E63" s="8" t="inlineStr">
         <is>
-          <t>line.price</t>
+          <t>col_price</t>
         </is>
       </c>
       <c r="F63" s="8" t="inlineStr">
         <is>
-          <t>line.total</t>
+          <t>col_total</t>
         </is>
       </c>
     </row>
@@ -1559,42 +1554,55 @@
       <c r="A64" s="8" t="n"/>
       <c r="B64" s="8" t="inlineStr">
         <is>
+          <t>DATA:*</t>
+        </is>
+      </c>
+      <c r="C64" s="8" t="inlineStr">
+        <is>
+          <t>line.item</t>
+        </is>
+      </c>
+      <c r="D64" s="8" t="inlineStr">
+        <is>
+          <t>line.qty</t>
+        </is>
+      </c>
+      <c r="E64" s="8" t="inlineStr">
+        <is>
+          <t>line.price</t>
+        </is>
+      </c>
+      <c r="F64" s="8" t="inlineStr">
+        <is>
+          <t>line.total</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="8" t="n"/>
+      <c r="B65" s="8" t="inlineStr">
+        <is>
           <t>FOOTER:1</t>
         </is>
       </c>
-      <c r="C64" s="8" t="inlineStr">
+      <c r="C65" s="8" t="inlineStr">
         <is>
           <t>footer.label</t>
         </is>
       </c>
-      <c r="D64" s="8" t="inlineStr">
+      <c r="D65" s="8" t="inlineStr">
         <is>
           <t>IGNORE</t>
         </is>
       </c>
-      <c r="E64" s="8" t="inlineStr">
+      <c r="E65" s="8" t="inlineStr">
         <is>
           <t>IGNORE</t>
         </is>
       </c>
-      <c r="F64" s="8" t="inlineStr">
+      <c r="F65" s="8" t="inlineStr">
         <is>
           <t>footer.value</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="1" t="inlineStr">
-        <is>
-          <t>doc:</t>
-        </is>
-      </c>
-      <c r="B65" s="1" t="inlineStr"/>
-      <c r="C65" s="1" t="inlineStr"/>
-      <c r="D65" s="1" t="inlineStr"/>
-      <c r="E65" s="1" t="inlineStr">
-        <is>
-          <t>HEADER/FOOTER are strict: wrong or missing value = no match.</t>
         </is>
       </c>
     </row>
@@ -1609,7 +1617,7 @@
       <c r="D66" s="1" t="inlineStr"/>
       <c r="E66" s="1" t="inlineStr">
         <is>
-          <t>DATA rows are lenient: wrong value emits a warning but extraction continues.</t>
+          <t>HEADER/FOOTER are strict: wrong or missing value = no match.</t>
         </is>
       </c>
     </row>
@@ -1624,7 +1632,7 @@
       <c r="D67" s="1" t="inlineStr"/>
       <c r="E67" s="1" t="inlineStr">
         <is>
-          <t>EMPTY column keyword: cell must be blank. IGNORE: consume without matching.</t>
+          <t>DATA rows are lenient: wrong value emits a warning but extraction continues.</t>
         </is>
       </c>
     </row>
@@ -1639,7 +1647,7 @@
       <c r="D68" s="1" t="inlineStr"/>
       <c r="E68" s="1" t="inlineStr">
         <is>
-          <t>── BOUNDED DATA + SKIP_IF (fixed-slot templates) ───────────────────────</t>
+          <t>EMPTY column keyword: cell must be blank. IGNORE: consume without matching.</t>
         </is>
       </c>
     </row>
@@ -1654,7 +1662,7 @@
       <c r="D69" s="1" t="inlineStr"/>
       <c r="E69" s="1" t="inlineStr">
         <is>
-          <t>Use DATA:{n,m} when the template pre-allocates a fixed number of rows.</t>
+          <t>── BOUNDED DATA + SKIP_IF (fixed-slot templates) ───────────────────────</t>
         </is>
       </c>
     </row>
@@ -1669,7 +1677,7 @@
       <c r="D70" s="1" t="inlineStr"/>
       <c r="E70" s="1" t="inlineStr">
         <is>
-          <t>n = min total physical rows expected, m = max total rows to scan.</t>
+          <t>Use DATA:{n,m} when the template pre-allocates a fixed number of rows.</t>
         </is>
       </c>
     </row>
@@ -1684,7 +1692,7 @@
       <c r="D71" s="1" t="inlineStr"/>
       <c r="E71" s="1" t="inlineStr">
         <is>
-          <t>SKIP_IF: rows matching the condition are silently excluded from output</t>
+          <t>n = min total physical rows expected, m = max total rows to scan.</t>
         </is>
       </c>
     </row>
@@ -1699,7 +1707,7 @@
       <c r="D72" s="1" t="inlineStr"/>
       <c r="E72" s="1" t="inlineStr">
         <is>
-          <t>but still count toward the {n,m} bounds.</t>
+          <t>SKIP_IF: rows matching the condition are silently excluded from output</t>
         </is>
       </c>
     </row>
@@ -1714,32 +1722,29 @@
       <c r="D73" s="1" t="inlineStr"/>
       <c r="E73" s="1" t="inlineStr">
         <is>
+          <t>but still count toward the {n,m} bounds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="1" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B74" s="1" t="inlineStr"/>
+      <c r="C74" s="1" t="inlineStr"/>
+      <c r="D74" s="1" t="inlineStr"/>
+      <c r="E74" s="1" t="inlineStr">
+        <is>
           <t>SKIP_IF is valid with DATA:{n,m} (rows count toward bounds) and DATA:* (rows filtered, scan continues).</t>
         </is>
       </c>
     </row>
-    <row r="74">
-      <c r="A74" s="7" t="inlineStr">
+    <row r="75">
+      <c r="A75" s="7" t="inlineStr">
         <is>
           <t>table:1</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="8" t="n"/>
-      <c r="B75" s="8" t="inlineStr">
-        <is>
-          <t>HEADER:1</t>
-        </is>
-      </c>
-      <c r="C75" s="8" t="inlineStr">
-        <is>
-          <t>col_item</t>
-        </is>
-      </c>
-      <c r="D75" s="8" t="inlineStr">
-        <is>
-          <t>col_qty</t>
         </is>
       </c>
     </row>
@@ -1747,17 +1752,17 @@
       <c r="A76" s="8" t="n"/>
       <c r="B76" s="8" t="inlineStr">
         <is>
-          <t>SKIP_IF</t>
+          <t>HEADER:1</t>
         </is>
       </c>
       <c r="C76" s="8" t="inlineStr">
         <is>
-          <t>EMPTY</t>
+          <t>col_item</t>
         </is>
       </c>
       <c r="D76" s="8" t="inlineStr">
         <is>
-          <t>IGNORE</t>
+          <t>col_qty</t>
         </is>
       </c>
     </row>
@@ -1765,17 +1770,17 @@
       <c r="A77" s="8" t="n"/>
       <c r="B77" s="8" t="inlineStr">
         <is>
-          <t>DATA:{0,15}</t>
+          <t>SKIP_IF</t>
         </is>
       </c>
       <c r="C77" s="8" t="inlineStr">
         <is>
-          <t>line.item</t>
+          <t>EMPTY</t>
         </is>
       </c>
       <c r="D77" s="8" t="inlineStr">
         <is>
-          <t>line.qty</t>
+          <t>IGNORE</t>
         </is>
       </c>
     </row>
@@ -1783,39 +1788,42 @@
       <c r="A78" s="8" t="n"/>
       <c r="B78" s="8" t="inlineStr">
         <is>
+          <t>DATA:{0,15}</t>
+        </is>
+      </c>
+      <c r="C78" s="8" t="inlineStr">
+        <is>
+          <t>line.item</t>
+        </is>
+      </c>
+      <c r="D78" s="8" t="inlineStr">
+        <is>
+          <t>line.qty</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="8" t="n"/>
+      <c r="B79" s="8" t="inlineStr">
+        <is>
           <t>FOOTER:1</t>
         </is>
       </c>
-      <c r="C78" s="8" t="inlineStr">
+      <c r="C79" s="8" t="inlineStr">
         <is>
           <t>lbl_total</t>
         </is>
       </c>
-      <c r="D78" s="8" t="inlineStr">
+      <c r="D79" s="8" t="inlineStr">
         <is>
           <t>inv.total</t>
         </is>
       </c>
     </row>
-    <row r="80">
-      <c r="A80" s="6" t="inlineStr">
+    <row r="81">
+      <c r="A81" s="6" t="inlineStr">
         <is>
           <t>END:</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="1" t="inlineStr">
-        <is>
-          <t>doc:</t>
-        </is>
-      </c>
-      <c r="B82" s="1" t="inlineStr"/>
-      <c r="C82" s="1" t="inlineStr"/>
-      <c r="D82" s="1" t="inlineStr"/>
-      <c r="E82" s="1" t="inlineStr">
-        <is>
-          <t>── QUICK REFERENCE ──────────────────────────────────────────────</t>
         </is>
       </c>
     </row>
@@ -1825,87 +1833,84 @@
           <t>doc:</t>
         </is>
       </c>
-      <c r="B83" s="1" t="inlineStr">
+      <c r="B83" s="1" t="inlineStr"/>
+      <c r="C83" s="1" t="inlineStr"/>
+      <c r="D83" s="1" t="inlineStr"/>
+      <c r="E83" s="1" t="inlineStr">
+        <is>
+          <t>── QUICK REFERENCE ──────────────────────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="1" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B84" s="1" t="inlineStr">
         <is>
           <t>doc: | free text</t>
         </is>
       </c>
-      <c r="C83" s="1" t="inlineStr"/>
-      <c r="D83" s="1" t="inlineStr">
+      <c r="C84" s="1" t="inlineStr"/>
+      <c r="D84" s="1" t="inlineStr">
         <is>
           <t>Inline comment. Ignored by engine.</t>
         </is>
       </c>
     </row>
-    <row r="84">
-      <c r="A84" s="3" t="inlineStr">
+    <row r="85">
+      <c r="A85" s="3" t="inlineStr">
         <is>
           <t>config:</t>
         </is>
       </c>
-      <c r="B84" s="3" t="inlineStr">
+      <c r="B85" s="3" t="inlineStr">
         <is>
           <t>config: | key | value</t>
         </is>
       </c>
-      <c r="C84" s="3" t="inlineStr"/>
-      <c r="D84" s="3" t="inlineStr">
+      <c r="C85" s="3" t="inlineStr"/>
+      <c r="D85" s="3" t="inlineStr">
         <is>
           <t>Global setting. Keys: read.direction, currency.sign, empty.aliases, ignore.case</t>
         </is>
       </c>
     </row>
-    <row r="85">
-      <c r="A85" s="4" t="inlineStr">
+    <row r="86">
+      <c r="A86" s="4" t="inlineStr">
         <is>
           <t>lbl:</t>
         </is>
       </c>
-      <c r="B85" s="4" t="inlineStr">
+      <c r="B86" s="4" t="inlineStr">
         <is>
           <t>lbl: | name | type | regex</t>
         </is>
       </c>
-      <c r="C85" s="4" t="inlineStr"/>
-      <c r="D85" s="4" t="inlineStr">
+      <c r="C86" s="4" t="inlineStr"/>
+      <c r="D86" s="4" t="inlineStr">
         <is>
           <t>Anchor label. Matched but never in output.</t>
         </is>
       </c>
     </row>
-    <row r="86">
-      <c r="A86" s="5" t="inlineStr">
+    <row r="87">
+      <c r="A87" s="5" t="inlineStr">
         <is>
           <t>var:</t>
         </is>
       </c>
-      <c r="B86" s="5" t="inlineStr">
+      <c r="B87" s="5" t="inlineStr">
         <is>
           <t>var: | name | type | regex</t>
         </is>
       </c>
-      <c r="C86" s="5" t="inlineStr"/>
-      <c r="D86" s="5" t="inlineStr">
+      <c r="C87" s="5" t="inlineStr"/>
+      <c r="D87" s="5" t="inlineStr">
         <is>
           <t>Extracted variable. Use dot notation for nesting.</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" t="inlineStr">
-        <is>
-          <t>cell:next</t>
-        </is>
-      </c>
-      <c r="B87" t="inlineStr">
-        <is>
-          <t>cell:next | FieldName</t>
-        </is>
-      </c>
-      <c r="C87" t="inlineStr"/>
-      <c r="D87" t="inlineStr">
-        <is>
-          <t>Read next non-empty cell (alias: cell:1).</t>
         </is>
       </c>
     </row>
@@ -1917,13 +1922,13 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>cell:next | IGNORE</t>
+          <t>cell:next | FieldName</t>
         </is>
       </c>
       <c r="C88" t="inlineStr"/>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Skip next non-empty cell without capturing.</t>
+          <t>Read next non-empty cell (alias: cell:1).</t>
         </is>
       </c>
     </row>
@@ -1935,155 +1940,173 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>cell:B5 | FieldName</t>
+          <t>cell:next | IGNORE</t>
         </is>
       </c>
       <c r="C89" t="inlineStr"/>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Jump directly to B5 (absolute reference). Ordering must be forward.</t>
+          <t>Skip next non-empty cell without capturing.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>seek:</t>
+          <t>cell:next</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>seek:G5</t>
+          <t>cell:B5 | FieldName</t>
         </is>
       </c>
       <c r="C90" t="inlineStr"/>
       <c r="D90" t="inlineStr">
         <is>
+          <t>Jump directly to B5 (absolute reference). Ordering must be forward.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>seek:</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>seek:G5</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr"/>
+      <c r="D91" t="inlineStr">
+        <is>
           <t>Reposition cursor to G5 without reading it. Resets abs-ref ordering constraint.</t>
         </is>
       </c>
     </row>
-    <row r="91">
-      <c r="A91" s="7" t="inlineStr">
+    <row r="92">
+      <c r="A92" s="7" t="inlineStr">
         <is>
           <t>table:*</t>
         </is>
       </c>
-      <c r="B91" s="7" t="inlineStr">
+      <c r="B92" s="7" t="inlineStr">
         <is>
           <t>table:*  (or table:1)</t>
         </is>
       </c>
-      <c r="C91" s="7" t="inlineStr"/>
-      <c r="D91" s="7" t="inlineStr">
+      <c r="C92" s="7" t="inlineStr"/>
+      <c r="D92" s="7" t="inlineStr">
         <is>
           <t>Begin a repeating table block.</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" s="8" t="inlineStr">
-        <is>
-          <t>HEADER:N</t>
-        </is>
-      </c>
-      <c r="B92" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> | HEADER:1 | F1 | F2</t>
-        </is>
-      </c>
-      <c r="C92" s="8" t="inlineStr"/>
-      <c r="D92" s="8" t="inlineStr">
-        <is>
-          <t>Strict header row template (col A must be blank).</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="8" t="inlineStr">
         <is>
-          <t>DATA:*</t>
+          <t>HEADER:N</t>
         </is>
       </c>
       <c r="B93" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | DATA:* | F1 | F2</t>
+          <t xml:space="preserve"> | HEADER:1 | F1 | F2</t>
         </is>
       </c>
       <c r="C93" s="8" t="inlineStr"/>
       <c r="D93" s="8" t="inlineStr">
         <is>
-          <t>Data row template (greedy, lenient validation).</t>
+          <t>Strict header row template (col A must be blank).</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="8" t="inlineStr">
         <is>
-          <t>DATA:{n,m}</t>
+          <t>DATA:*</t>
         </is>
       </c>
       <c r="B94" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | DATA:{0,15} | F1 | F2</t>
+          <t xml:space="preserve"> | DATA:* | F1 | F2</t>
         </is>
       </c>
       <c r="C94" s="8" t="inlineStr"/>
       <c r="D94" s="8" t="inlineStr">
         <is>
+          <t>Data row template (greedy, lenient validation).</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="8" t="inlineStr">
+        <is>
+          <t>DATA:{n,m}</t>
+        </is>
+      </c>
+      <c r="B95" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> | DATA:{0,15} | F1 | F2</t>
+        </is>
+      </c>
+      <c r="C95" s="8" t="inlineStr"/>
+      <c r="D95" s="8" t="inlineStr">
+        <is>
           <t>Bounded data: scan at most m physical rows, warn if &lt; n.</t>
         </is>
       </c>
     </row>
-    <row r="95">
-      <c r="A95" t="inlineStr">
+    <row r="96">
+      <c r="A96" t="inlineStr">
         <is>
           <t>SKIP_IF</t>
         </is>
       </c>
-      <c r="B95" t="inlineStr">
+      <c r="B96" t="inlineStr">
         <is>
           <t xml:space="preserve"> | SKIP_IF | EMPTY | IGNORE</t>
         </is>
       </c>
-      <c r="C95" t="inlineStr"/>
-      <c r="D95" t="inlineStr">
+      <c r="C96" t="inlineStr"/>
+      <c r="D96" t="inlineStr">
         <is>
           <t>Skip row if non-IGNORE columns match. Valid with DATA:{n,m} and DATA:*.</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" s="8" t="inlineStr">
-        <is>
-          <t>FOOTER:N</t>
-        </is>
-      </c>
-      <c r="B96" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> | FOOTER:1 | F1 | F2</t>
-        </is>
-      </c>
-      <c r="C96" s="8" t="inlineStr"/>
-      <c r="D96" s="8" t="inlineStr">
-        <is>
-          <t>Strict footer row template.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="8" t="inlineStr">
         <is>
-          <t>SPLITTER</t>
+          <t>FOOTER:N</t>
         </is>
       </c>
       <c r="B97" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | SPLITTER:1</t>
+          <t xml:space="preserve"> | FOOTER:1 | F1 | F2</t>
         </is>
       </c>
       <c r="C97" s="8" t="inlineStr"/>
       <c r="D97" s="8" t="inlineStr">
+        <is>
+          <t>Strict footer row template.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="8" t="inlineStr">
+        <is>
+          <t>SPLITTER</t>
+        </is>
+      </c>
+      <c r="B98" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> | SPLITTER:1</t>
+        </is>
+      </c>
+      <c r="C98" s="8" t="inlineStr"/>
+      <c r="D98" s="8" t="inlineStr">
         <is>
           <t>All columns must be blank (separator row).</t>
         </is>

</xml_diff>

<commit_message>
docs: document column-A modifier syntax (not-null, var:glob, var:literal, lbl:re)
- docs/pattern-file.md: new 'Column A modifiers' subsection with table,
  examples, and semantics for var:glob/literal/re, not-null/not-empty,
  and order-independent combinations; update column A table and lbl:/var:
  descriptions; add lbl:re alias mention
- README.md: new 'Optional quality gates' subsection with quick-reference
  table and code example
- CHANGELOG.md: add modifier syntax entry under [Unreleased]
- grepxcel/docs_generator.py: add modifier example rows (not-null, glob,
  literal, lbl:not-null) to the VAR section of pattern-reference.xlsx
- docs/pattern-reference.xlsx: regenerated with new modifier examples

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K6EyxWBecbqyp9uRx7c4J8
</commit_message>
<xml_diff>
--- a/docs/pattern-reference.xlsx
+++ b/docs/pattern-reference.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F98"/>
+  <dimension ref="A1:F109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1251,7 +1251,7 @@
       <c r="D44" s="1" t="inlineStr"/>
       <c r="E44" s="1" t="inlineStr">
         <is>
-          <t>Everything between START: and END: defines the extraction order.</t>
+          <t>Column A modifiers — order-independent, colon-separated. Add after var: or lbl:</t>
         </is>
       </c>
     </row>
@@ -1266,7 +1266,7 @@
       <c r="D45" s="1" t="inlineStr"/>
       <c r="E45" s="1" t="inlineStr">
         <is>
-          <t>cell:next  reads the next non-empty cell (alias: cell:1). Scans in read.direction order.</t>
+          <t>not-null / not-empty (synonyms): fatal error if value is empty/null (always, not just with --strict)</t>
         </is>
       </c>
     </row>
@@ -1281,7 +1281,7 @@
       <c r="D46" s="1" t="inlineStr"/>
       <c r="E46" s="1" t="inlineStr">
         <is>
-          <t>cell:B5    jumps directly to cell B5 (absolute A1-notation reference).</t>
+          <t>var:glob → column D is a shell glob (PROD-* matches PROD-42); type check still runs</t>
         </is>
       </c>
     </row>
@@ -1296,7 +1296,7 @@
       <c r="D47" s="1" t="inlineStr"/>
       <c r="E47" s="1" t="inlineStr">
         <is>
-          <t>seek:G5    repositions the cursor to G5 WITHOUT reading it. Next cell:next starts from there.</t>
+          <t>var:literal → column D is exact string (special chars are literal, not regex)</t>
         </is>
       </c>
     </row>
@@ -1311,7 +1311,7 @@
       <c r="D48" s="1" t="inlineStr"/>
       <c r="E48" s="1" t="inlineStr">
         <is>
-          <t>dir:LR     switches scan direction to left-to-right from here on (dir:TD = top-down).</t>
+          <t>var:re → explicit alias for default regex mode; lbl:re → alias for lbl:regexp</t>
         </is>
       </c>
     </row>
@@ -1326,128 +1326,145 @@
       <c r="D49" s="1" t="inlineStr"/>
       <c r="E49" s="1" t="inlineStr">
         <is>
-          <t>table:*    finds all instances of a repeating table block.</t>
+          <t>Modifiers combine freely: var:not-null:glob, lbl:not-null, var:literal:not-empty</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="6" t="inlineStr">
-        <is>
-          <t>START:</t>
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>var:not-null</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>invoice.number</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>INV-\d+</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>Required regex field — fatal if empty.</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="7" t="inlineStr">
-        <is>
-          <t>cell:A1</t>
-        </is>
-      </c>
-      <c r="B51" s="7" t="inlineStr">
-        <is>
-          <t>po_label</t>
-        </is>
-      </c>
-      <c r="C51" s="7" t="inlineStr"/>
-      <c r="D51" s="7" t="inlineStr"/>
-      <c r="E51" s="7" t="inlineStr">
-        <is>
-          <t>Jump to A1 and read "PO Number:" anchor (lbl: field — not in output).</t>
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>var:glob</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>sku</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>PROD-*</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>Glob match: PROD-42, PROD-XYZ, ...</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="7" t="inlineStr">
-        <is>
-          <t>cell:next</t>
-        </is>
-      </c>
-      <c r="B52" s="7" t="inlineStr">
-        <is>
-          <t>po.number</t>
-        </is>
-      </c>
-      <c r="C52" s="7" t="inlineStr"/>
-      <c r="D52" s="7" t="inlineStr"/>
-      <c r="E52" s="7" t="inlineStr">
-        <is>
-          <t>Read next non-empty cell after A1 → the PO number.</t>
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>var:literal</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>Exact string match — "Active" only.</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="7" t="inlineStr">
-        <is>
-          <t>cell:C1</t>
-        </is>
-      </c>
-      <c r="B53" s="7" t="inlineStr">
-        <is>
-          <t>date_label</t>
-        </is>
-      </c>
-      <c r="C53" s="7" t="inlineStr"/>
-      <c r="D53" s="7" t="inlineStr"/>
-      <c r="E53" s="7" t="inlineStr">
-        <is>
-          <t>Jump to C1 and read "Date:" anchor.</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="7" t="inlineStr">
-        <is>
-          <t>cell:next</t>
-        </is>
-      </c>
-      <c r="B54" s="7" t="inlineStr">
-        <is>
-          <t>po.date</t>
-        </is>
-      </c>
-      <c r="C54" s="7" t="inlineStr"/>
-      <c r="D54" s="7" t="inlineStr"/>
-      <c r="E54" s="7" t="inlineStr">
-        <is>
-          <t>Read next non-empty cell after C1 → the PO date.</t>
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>lbl:not-null</t>
+        </is>
+      </c>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>inv_label</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D53" s="4" t="inlineStr">
+        <is>
+          <t>Invoice:</t>
+        </is>
+      </c>
+      <c r="E53" s="4" t="inlineStr">
+        <is>
+          <t>Anchor must be present or fatal.</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="7" t="inlineStr">
-        <is>
-          <t>cell:next</t>
-        </is>
-      </c>
-      <c r="B55" s="7" t="inlineStr">
-        <is>
-          <t>vendor_label</t>
-        </is>
-      </c>
-      <c r="C55" s="7" t="inlineStr"/>
-      <c r="D55" s="7" t="inlineStr"/>
-      <c r="E55" s="7" t="inlineStr">
-        <is>
-          <t>Read next non-empty cell → "Vendor:" anchor.</t>
+      <c r="A55" s="1" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B55" s="1" t="inlineStr"/>
+      <c r="C55" s="1" t="inlineStr"/>
+      <c r="D55" s="1" t="inlineStr"/>
+      <c r="E55" s="1" t="inlineStr">
+        <is>
+          <t>Everything between START: and END: defines the extraction order.</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="7" t="inlineStr">
-        <is>
-          <t>cell:next</t>
-        </is>
-      </c>
-      <c r="B56" s="7" t="inlineStr">
-        <is>
-          <t>vendor.name</t>
-        </is>
-      </c>
-      <c r="C56" s="7" t="inlineStr"/>
-      <c r="D56" s="7" t="inlineStr"/>
-      <c r="E56" s="7" t="inlineStr">
-        <is>
-          <t>Extract the vendor name.</t>
+      <c r="A56" s="1" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B56" s="1" t="inlineStr"/>
+      <c r="C56" s="1" t="inlineStr"/>
+      <c r="D56" s="1" t="inlineStr"/>
+      <c r="E56" s="1" t="inlineStr">
+        <is>
+          <t>cell:next  reads the next non-empty cell (alias: cell:1). Scans in read.direction order.</t>
         </is>
       </c>
     </row>
@@ -1462,26 +1479,37 @@
       <c r="D57" s="1" t="inlineStr"/>
       <c r="E57" s="1" t="inlineStr">
         <is>
-          <t>Use IGNORE to skip a non-empty cell without defining a field for it.</t>
+          <t>cell:B5    jumps directly to cell B5 (absolute A1-notation reference).</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="7" t="inlineStr">
-        <is>
-          <t>cell:next</t>
-        </is>
-      </c>
-      <c r="B58" s="7" t="inlineStr">
-        <is>
-          <t>IGNORE</t>
-        </is>
-      </c>
-      <c r="C58" s="7" t="inlineStr"/>
-      <c r="D58" s="7" t="inlineStr"/>
-      <c r="E58" s="7" t="inlineStr">
-        <is>
-          <t>Skip one non-empty cell without capturing it.</t>
+      <c r="A58" s="1" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B58" s="1" t="inlineStr"/>
+      <c r="C58" s="1" t="inlineStr"/>
+      <c r="D58" s="1" t="inlineStr"/>
+      <c r="E58" s="1" t="inlineStr">
+        <is>
+          <t>seek:G5    repositions the cursor to G5 WITHOUT reading it. Next cell:next starts from there.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="1" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B59" s="1" t="inlineStr"/>
+      <c r="C59" s="1" t="inlineStr"/>
+      <c r="D59" s="1" t="inlineStr"/>
+      <c r="E59" s="1" t="inlineStr">
+        <is>
+          <t>dir:LR     switches scan direction to left-to-right from here on (dir:TD = top-down).</t>
         </is>
       </c>
     </row>
@@ -1496,143 +1524,128 @@
       <c r="D60" s="1" t="inlineStr"/>
       <c r="E60" s="1" t="inlineStr">
         <is>
-          <t>table:* matches 0-or-more mini-table instances in greedy order.</t>
+          <t>table:*    finds all instances of a repeating table block.</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="1" t="inlineStr">
-        <is>
-          <t>doc:</t>
-        </is>
-      </c>
-      <c r="B61" s="1" t="inlineStr"/>
-      <c r="C61" s="1" t="inlineStr"/>
-      <c r="D61" s="1" t="inlineStr"/>
-      <c r="E61" s="1" t="inlineStr">
-        <is>
-          <t>Use table:1 when exactly one instance is expected.</t>
+      <c r="A61" s="6" t="inlineStr">
+        <is>
+          <t>START:</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
         <is>
-          <t>table:*</t>
+          <t>cell:A1</t>
+        </is>
+      </c>
+      <c r="B62" s="7" t="inlineStr">
+        <is>
+          <t>po_label</t>
+        </is>
+      </c>
+      <c r="C62" s="7" t="inlineStr"/>
+      <c r="D62" s="7" t="inlineStr"/>
+      <c r="E62" s="7" t="inlineStr">
+        <is>
+          <t>Jump to A1 and read "PO Number:" anchor (lbl: field — not in output).</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="8" t="n"/>
-      <c r="B63" s="8" t="inlineStr">
-        <is>
-          <t>HEADER:1</t>
-        </is>
-      </c>
-      <c r="C63" s="8" t="inlineStr">
-        <is>
-          <t>col_item</t>
-        </is>
-      </c>
-      <c r="D63" s="8" t="inlineStr">
-        <is>
-          <t>col_qty</t>
-        </is>
-      </c>
-      <c r="E63" s="8" t="inlineStr">
-        <is>
-          <t>col_price</t>
-        </is>
-      </c>
-      <c r="F63" s="8" t="inlineStr">
-        <is>
-          <t>col_total</t>
+      <c r="A63" s="7" t="inlineStr">
+        <is>
+          <t>cell:next</t>
+        </is>
+      </c>
+      <c r="B63" s="7" t="inlineStr">
+        <is>
+          <t>po.number</t>
+        </is>
+      </c>
+      <c r="C63" s="7" t="inlineStr"/>
+      <c r="D63" s="7" t="inlineStr"/>
+      <c r="E63" s="7" t="inlineStr">
+        <is>
+          <t>Read next non-empty cell after A1 → the PO number.</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="8" t="n"/>
-      <c r="B64" s="8" t="inlineStr">
-        <is>
-          <t>DATA:*</t>
-        </is>
-      </c>
-      <c r="C64" s="8" t="inlineStr">
-        <is>
-          <t>line.item</t>
-        </is>
-      </c>
-      <c r="D64" s="8" t="inlineStr">
-        <is>
-          <t>line.qty</t>
-        </is>
-      </c>
-      <c r="E64" s="8" t="inlineStr">
-        <is>
-          <t>line.price</t>
-        </is>
-      </c>
-      <c r="F64" s="8" t="inlineStr">
-        <is>
-          <t>line.total</t>
+      <c r="A64" s="7" t="inlineStr">
+        <is>
+          <t>cell:C1</t>
+        </is>
+      </c>
+      <c r="B64" s="7" t="inlineStr">
+        <is>
+          <t>date_label</t>
+        </is>
+      </c>
+      <c r="C64" s="7" t="inlineStr"/>
+      <c r="D64" s="7" t="inlineStr"/>
+      <c r="E64" s="7" t="inlineStr">
+        <is>
+          <t>Jump to C1 and read "Date:" anchor.</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="8" t="n"/>
-      <c r="B65" s="8" t="inlineStr">
-        <is>
-          <t>FOOTER:1</t>
-        </is>
-      </c>
-      <c r="C65" s="8" t="inlineStr">
-        <is>
-          <t>footer.label</t>
-        </is>
-      </c>
-      <c r="D65" s="8" t="inlineStr">
-        <is>
-          <t>IGNORE</t>
-        </is>
-      </c>
-      <c r="E65" s="8" t="inlineStr">
-        <is>
-          <t>IGNORE</t>
-        </is>
-      </c>
-      <c r="F65" s="8" t="inlineStr">
-        <is>
-          <t>footer.value</t>
+      <c r="A65" s="7" t="inlineStr">
+        <is>
+          <t>cell:next</t>
+        </is>
+      </c>
+      <c r="B65" s="7" t="inlineStr">
+        <is>
+          <t>po.date</t>
+        </is>
+      </c>
+      <c r="C65" s="7" t="inlineStr"/>
+      <c r="D65" s="7" t="inlineStr"/>
+      <c r="E65" s="7" t="inlineStr">
+        <is>
+          <t>Read next non-empty cell after C1 → the PO date.</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="1" t="inlineStr">
-        <is>
-          <t>doc:</t>
-        </is>
-      </c>
-      <c r="B66" s="1" t="inlineStr"/>
-      <c r="C66" s="1" t="inlineStr"/>
-      <c r="D66" s="1" t="inlineStr"/>
-      <c r="E66" s="1" t="inlineStr">
-        <is>
-          <t>HEADER/FOOTER are strict: wrong or missing value = no match.</t>
+      <c r="A66" s="7" t="inlineStr">
+        <is>
+          <t>cell:next</t>
+        </is>
+      </c>
+      <c r="B66" s="7" t="inlineStr">
+        <is>
+          <t>vendor_label</t>
+        </is>
+      </c>
+      <c r="C66" s="7" t="inlineStr"/>
+      <c r="D66" s="7" t="inlineStr"/>
+      <c r="E66" s="7" t="inlineStr">
+        <is>
+          <t>Read next non-empty cell → "Vendor:" anchor.</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="1" t="inlineStr">
-        <is>
-          <t>doc:</t>
-        </is>
-      </c>
-      <c r="B67" s="1" t="inlineStr"/>
-      <c r="C67" s="1" t="inlineStr"/>
-      <c r="D67" s="1" t="inlineStr"/>
-      <c r="E67" s="1" t="inlineStr">
-        <is>
-          <t>DATA rows are lenient: wrong value emits a warning but extraction continues.</t>
+      <c r="A67" s="7" t="inlineStr">
+        <is>
+          <t>cell:next</t>
+        </is>
+      </c>
+      <c r="B67" s="7" t="inlineStr">
+        <is>
+          <t>vendor.name</t>
+        </is>
+      </c>
+      <c r="C67" s="7" t="inlineStr"/>
+      <c r="D67" s="7" t="inlineStr"/>
+      <c r="E67" s="7" t="inlineStr">
+        <is>
+          <t>Extract the vendor name.</t>
         </is>
       </c>
     </row>
@@ -1647,37 +1660,26 @@
       <c r="D68" s="1" t="inlineStr"/>
       <c r="E68" s="1" t="inlineStr">
         <is>
-          <t>EMPTY column keyword: cell must be blank. IGNORE: consume without matching.</t>
+          <t>Use IGNORE to skip a non-empty cell without defining a field for it.</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="1" t="inlineStr">
-        <is>
-          <t>doc:</t>
-        </is>
-      </c>
-      <c r="B69" s="1" t="inlineStr"/>
-      <c r="C69" s="1" t="inlineStr"/>
-      <c r="D69" s="1" t="inlineStr"/>
-      <c r="E69" s="1" t="inlineStr">
-        <is>
-          <t>── BOUNDED DATA + SKIP_IF (fixed-slot templates) ───────────────────────</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="1" t="inlineStr">
-        <is>
-          <t>doc:</t>
-        </is>
-      </c>
-      <c r="B70" s="1" t="inlineStr"/>
-      <c r="C70" s="1" t="inlineStr"/>
-      <c r="D70" s="1" t="inlineStr"/>
-      <c r="E70" s="1" t="inlineStr">
-        <is>
-          <t>Use DATA:{n,m} when the template pre-allocates a fixed number of rows.</t>
+      <c r="A69" s="7" t="inlineStr">
+        <is>
+          <t>cell:next</t>
+        </is>
+      </c>
+      <c r="B69" s="7" t="inlineStr">
+        <is>
+          <t>IGNORE</t>
+        </is>
+      </c>
+      <c r="C69" s="7" t="inlineStr"/>
+      <c r="D69" s="7" t="inlineStr"/>
+      <c r="E69" s="7" t="inlineStr">
+        <is>
+          <t>Skip one non-empty cell without capturing it.</t>
         </is>
       </c>
     </row>
@@ -1692,7 +1694,7 @@
       <c r="D71" s="1" t="inlineStr"/>
       <c r="E71" s="1" t="inlineStr">
         <is>
-          <t>n = min total physical rows expected, m = max total rows to scan.</t>
+          <t>table:* matches 0-or-more mini-table instances in greedy order.</t>
         </is>
       </c>
     </row>
@@ -1707,44 +1709,70 @@
       <c r="D72" s="1" t="inlineStr"/>
       <c r="E72" s="1" t="inlineStr">
         <is>
-          <t>SKIP_IF: rows matching the condition are silently excluded from output</t>
+          <t>Use table:1 when exactly one instance is expected.</t>
         </is>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="1" t="inlineStr">
-        <is>
-          <t>doc:</t>
-        </is>
-      </c>
-      <c r="B73" s="1" t="inlineStr"/>
-      <c r="C73" s="1" t="inlineStr"/>
-      <c r="D73" s="1" t="inlineStr"/>
-      <c r="E73" s="1" t="inlineStr">
-        <is>
-          <t>but still count toward the {n,m} bounds.</t>
+      <c r="A73" s="7" t="inlineStr">
+        <is>
+          <t>table:*</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="1" t="inlineStr">
-        <is>
-          <t>doc:</t>
-        </is>
-      </c>
-      <c r="B74" s="1" t="inlineStr"/>
-      <c r="C74" s="1" t="inlineStr"/>
-      <c r="D74" s="1" t="inlineStr"/>
-      <c r="E74" s="1" t="inlineStr">
-        <is>
-          <t>SKIP_IF is valid with DATA:{n,m} (rows count toward bounds) and DATA:* (rows filtered, scan continues).</t>
+      <c r="A74" s="8" t="n"/>
+      <c r="B74" s="8" t="inlineStr">
+        <is>
+          <t>HEADER:1</t>
+        </is>
+      </c>
+      <c r="C74" s="8" t="inlineStr">
+        <is>
+          <t>col_item</t>
+        </is>
+      </c>
+      <c r="D74" s="8" t="inlineStr">
+        <is>
+          <t>col_qty</t>
+        </is>
+      </c>
+      <c r="E74" s="8" t="inlineStr">
+        <is>
+          <t>col_price</t>
+        </is>
+      </c>
+      <c r="F74" s="8" t="inlineStr">
+        <is>
+          <t>col_total</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="7" t="inlineStr">
-        <is>
-          <t>table:1</t>
+      <c r="A75" s="8" t="n"/>
+      <c r="B75" s="8" t="inlineStr">
+        <is>
+          <t>DATA:*</t>
+        </is>
+      </c>
+      <c r="C75" s="8" t="inlineStr">
+        <is>
+          <t>line.item</t>
+        </is>
+      </c>
+      <c r="D75" s="8" t="inlineStr">
+        <is>
+          <t>line.qty</t>
+        </is>
+      </c>
+      <c r="E75" s="8" t="inlineStr">
+        <is>
+          <t>line.price</t>
+        </is>
+      </c>
+      <c r="F75" s="8" t="inlineStr">
+        <is>
+          <t>line.total</t>
         </is>
       </c>
     </row>
@@ -1752,78 +1780,117 @@
       <c r="A76" s="8" t="n"/>
       <c r="B76" s="8" t="inlineStr">
         <is>
-          <t>HEADER:1</t>
+          <t>FOOTER:1</t>
         </is>
       </c>
       <c r="C76" s="8" t="inlineStr">
         <is>
-          <t>col_item</t>
+          <t>footer.label</t>
         </is>
       </c>
       <c r="D76" s="8" t="inlineStr">
         <is>
-          <t>col_qty</t>
+          <t>IGNORE</t>
+        </is>
+      </c>
+      <c r="E76" s="8" t="inlineStr">
+        <is>
+          <t>IGNORE</t>
+        </is>
+      </c>
+      <c r="F76" s="8" t="inlineStr">
+        <is>
+          <t>footer.value</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="8" t="n"/>
-      <c r="B77" s="8" t="inlineStr">
-        <is>
-          <t>SKIP_IF</t>
-        </is>
-      </c>
-      <c r="C77" s="8" t="inlineStr">
-        <is>
-          <t>EMPTY</t>
-        </is>
-      </c>
-      <c r="D77" s="8" t="inlineStr">
-        <is>
-          <t>IGNORE</t>
+      <c r="A77" s="1" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B77" s="1" t="inlineStr"/>
+      <c r="C77" s="1" t="inlineStr"/>
+      <c r="D77" s="1" t="inlineStr"/>
+      <c r="E77" s="1" t="inlineStr">
+        <is>
+          <t>HEADER/FOOTER are strict: wrong or missing value = no match.</t>
         </is>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="8" t="n"/>
-      <c r="B78" s="8" t="inlineStr">
-        <is>
-          <t>DATA:{0,15}</t>
-        </is>
-      </c>
-      <c r="C78" s="8" t="inlineStr">
-        <is>
-          <t>line.item</t>
-        </is>
-      </c>
-      <c r="D78" s="8" t="inlineStr">
-        <is>
-          <t>line.qty</t>
+      <c r="A78" s="1" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B78" s="1" t="inlineStr"/>
+      <c r="C78" s="1" t="inlineStr"/>
+      <c r="D78" s="1" t="inlineStr"/>
+      <c r="E78" s="1" t="inlineStr">
+        <is>
+          <t>DATA rows are lenient: wrong value emits a warning but extraction continues.</t>
         </is>
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="8" t="n"/>
-      <c r="B79" s="8" t="inlineStr">
-        <is>
-          <t>FOOTER:1</t>
-        </is>
-      </c>
-      <c r="C79" s="8" t="inlineStr">
-        <is>
-          <t>lbl_total</t>
-        </is>
-      </c>
-      <c r="D79" s="8" t="inlineStr">
-        <is>
-          <t>inv.total</t>
+      <c r="A79" s="1" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B79" s="1" t="inlineStr"/>
+      <c r="C79" s="1" t="inlineStr"/>
+      <c r="D79" s="1" t="inlineStr"/>
+      <c r="E79" s="1" t="inlineStr">
+        <is>
+          <t>EMPTY column keyword: cell must be blank. IGNORE: consume without matching.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="1" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B80" s="1" t="inlineStr"/>
+      <c r="C80" s="1" t="inlineStr"/>
+      <c r="D80" s="1" t="inlineStr"/>
+      <c r="E80" s="1" t="inlineStr">
+        <is>
+          <t>── BOUNDED DATA + SKIP_IF (fixed-slot templates) ───────────────────────</t>
         </is>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="6" t="inlineStr">
-        <is>
-          <t>END:</t>
+      <c r="A81" s="1" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B81" s="1" t="inlineStr"/>
+      <c r="C81" s="1" t="inlineStr"/>
+      <c r="D81" s="1" t="inlineStr"/>
+      <c r="E81" s="1" t="inlineStr">
+        <is>
+          <t>Use DATA:{n,m} when the template pre-allocates a fixed number of rows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="1" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B82" s="1" t="inlineStr"/>
+      <c r="C82" s="1" t="inlineStr"/>
+      <c r="D82" s="1" t="inlineStr"/>
+      <c r="E82" s="1" t="inlineStr">
+        <is>
+          <t>n = min total physical rows expected, m = max total rows to scan.</t>
         </is>
       </c>
     </row>
@@ -1838,7 +1905,7 @@
       <c r="D83" s="1" t="inlineStr"/>
       <c r="E83" s="1" t="inlineStr">
         <is>
-          <t>── QUICK REFERENCE ──────────────────────────────────────────────</t>
+          <t>SKIP_IF: rows matching the condition are silently excluded from output</t>
         </is>
       </c>
     </row>
@@ -1848,265 +1915,396 @@
           <t>doc:</t>
         </is>
       </c>
-      <c r="B84" s="1" t="inlineStr">
+      <c r="B84" s="1" t="inlineStr"/>
+      <c r="C84" s="1" t="inlineStr"/>
+      <c r="D84" s="1" t="inlineStr"/>
+      <c r="E84" s="1" t="inlineStr">
+        <is>
+          <t>but still count toward the {n,m} bounds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="1" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B85" s="1" t="inlineStr"/>
+      <c r="C85" s="1" t="inlineStr"/>
+      <c r="D85" s="1" t="inlineStr"/>
+      <c r="E85" s="1" t="inlineStr">
+        <is>
+          <t>SKIP_IF is valid with DATA:{n,m} (rows count toward bounds) and DATA:* (rows filtered, scan continues).</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="7" t="inlineStr">
+        <is>
+          <t>table:1</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="8" t="n"/>
+      <c r="B87" s="8" t="inlineStr">
+        <is>
+          <t>HEADER:1</t>
+        </is>
+      </c>
+      <c r="C87" s="8" t="inlineStr">
+        <is>
+          <t>col_item</t>
+        </is>
+      </c>
+      <c r="D87" s="8" t="inlineStr">
+        <is>
+          <t>col_qty</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="8" t="n"/>
+      <c r="B88" s="8" t="inlineStr">
+        <is>
+          <t>SKIP_IF</t>
+        </is>
+      </c>
+      <c r="C88" s="8" t="inlineStr">
+        <is>
+          <t>EMPTY</t>
+        </is>
+      </c>
+      <c r="D88" s="8" t="inlineStr">
+        <is>
+          <t>IGNORE</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="8" t="n"/>
+      <c r="B89" s="8" t="inlineStr">
+        <is>
+          <t>DATA:{0,15}</t>
+        </is>
+      </c>
+      <c r="C89" s="8" t="inlineStr">
+        <is>
+          <t>line.item</t>
+        </is>
+      </c>
+      <c r="D89" s="8" t="inlineStr">
+        <is>
+          <t>line.qty</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="8" t="n"/>
+      <c r="B90" s="8" t="inlineStr">
+        <is>
+          <t>FOOTER:1</t>
+        </is>
+      </c>
+      <c r="C90" s="8" t="inlineStr">
+        <is>
+          <t>lbl_total</t>
+        </is>
+      </c>
+      <c r="D90" s="8" t="inlineStr">
+        <is>
+          <t>inv.total</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="6" t="inlineStr">
+        <is>
+          <t>END:</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="1" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B94" s="1" t="inlineStr"/>
+      <c r="C94" s="1" t="inlineStr"/>
+      <c r="D94" s="1" t="inlineStr"/>
+      <c r="E94" s="1" t="inlineStr">
+        <is>
+          <t>── QUICK REFERENCE ──────────────────────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="1" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B95" s="1" t="inlineStr">
         <is>
           <t>doc: | free text</t>
         </is>
       </c>
-      <c r="C84" s="1" t="inlineStr"/>
-      <c r="D84" s="1" t="inlineStr">
+      <c r="C95" s="1" t="inlineStr"/>
+      <c r="D95" s="1" t="inlineStr">
         <is>
           <t>Inline comment. Ignored by engine.</t>
         </is>
       </c>
     </row>
-    <row r="85">
-      <c r="A85" s="3" t="inlineStr">
+    <row r="96">
+      <c r="A96" s="3" t="inlineStr">
         <is>
           <t>config:</t>
         </is>
       </c>
-      <c r="B85" s="3" t="inlineStr">
+      <c r="B96" s="3" t="inlineStr">
         <is>
           <t>config: | key | value</t>
         </is>
       </c>
-      <c r="C85" s="3" t="inlineStr"/>
-      <c r="D85" s="3" t="inlineStr">
+      <c r="C96" s="3" t="inlineStr"/>
+      <c r="D96" s="3" t="inlineStr">
         <is>
           <t>Global setting. Keys: read.direction, currency.sign, empty.aliases, ignore.case</t>
         </is>
       </c>
     </row>
-    <row r="86">
-      <c r="A86" s="4" t="inlineStr">
+    <row r="97">
+      <c r="A97" s="4" t="inlineStr">
         <is>
           <t>lbl:</t>
         </is>
       </c>
-      <c r="B86" s="4" t="inlineStr">
+      <c r="B97" s="4" t="inlineStr">
         <is>
           <t>lbl: | name | type | regex</t>
         </is>
       </c>
-      <c r="C86" s="4" t="inlineStr"/>
-      <c r="D86" s="4" t="inlineStr">
+      <c r="C97" s="4" t="inlineStr"/>
+      <c r="D97" s="4" t="inlineStr">
         <is>
           <t>Anchor label. Matched but never in output.</t>
         </is>
       </c>
     </row>
-    <row r="87">
-      <c r="A87" s="5" t="inlineStr">
+    <row r="98">
+      <c r="A98" s="5" t="inlineStr">
         <is>
           <t>var:</t>
         </is>
       </c>
-      <c r="B87" s="5" t="inlineStr">
+      <c r="B98" s="5" t="inlineStr">
         <is>
           <t>var: | name | type | regex</t>
         </is>
       </c>
-      <c r="C87" s="5" t="inlineStr"/>
-      <c r="D87" s="5" t="inlineStr">
+      <c r="C98" s="5" t="inlineStr"/>
+      <c r="D98" s="5" t="inlineStr">
         <is>
           <t>Extracted variable. Use dot notation for nesting.</t>
         </is>
       </c>
     </row>
-    <row r="88">
-      <c r="A88" t="inlineStr">
+    <row r="99">
+      <c r="A99" t="inlineStr">
         <is>
           <t>cell:next</t>
         </is>
       </c>
-      <c r="B88" t="inlineStr">
+      <c r="B99" t="inlineStr">
         <is>
           <t>cell:next | FieldName</t>
         </is>
       </c>
-      <c r="C88" t="inlineStr"/>
-      <c r="D88" t="inlineStr">
+      <c r="C99" t="inlineStr"/>
+      <c r="D99" t="inlineStr">
         <is>
           <t>Read next non-empty cell (alias: cell:1).</t>
         </is>
       </c>
     </row>
-    <row r="89">
-      <c r="A89" t="inlineStr">
+    <row r="100">
+      <c r="A100" t="inlineStr">
         <is>
           <t>cell:next</t>
         </is>
       </c>
-      <c r="B89" t="inlineStr">
+      <c r="B100" t="inlineStr">
         <is>
           <t>cell:next | IGNORE</t>
         </is>
       </c>
-      <c r="C89" t="inlineStr"/>
-      <c r="D89" t="inlineStr">
+      <c r="C100" t="inlineStr"/>
+      <c r="D100" t="inlineStr">
         <is>
           <t>Skip next non-empty cell without capturing.</t>
         </is>
       </c>
     </row>
-    <row r="90">
-      <c r="A90" t="inlineStr">
+    <row r="101">
+      <c r="A101" t="inlineStr">
         <is>
           <t>cell:next</t>
         </is>
       </c>
-      <c r="B90" t="inlineStr">
+      <c r="B101" t="inlineStr">
         <is>
           <t>cell:B5 | FieldName</t>
         </is>
       </c>
-      <c r="C90" t="inlineStr"/>
-      <c r="D90" t="inlineStr">
+      <c r="C101" t="inlineStr"/>
+      <c r="D101" t="inlineStr">
         <is>
           <t>Jump directly to B5 (absolute reference). Ordering must be forward.</t>
         </is>
       </c>
     </row>
-    <row r="91">
-      <c r="A91" t="inlineStr">
+    <row r="102">
+      <c r="A102" t="inlineStr">
         <is>
           <t>seek:</t>
         </is>
       </c>
-      <c r="B91" t="inlineStr">
+      <c r="B102" t="inlineStr">
         <is>
           <t>seek:G5</t>
         </is>
       </c>
-      <c r="C91" t="inlineStr"/>
-      <c r="D91" t="inlineStr">
+      <c r="C102" t="inlineStr"/>
+      <c r="D102" t="inlineStr">
         <is>
           <t>Reposition cursor to G5 without reading it. Resets abs-ref ordering constraint.</t>
         </is>
       </c>
     </row>
-    <row r="92">
-      <c r="A92" s="7" t="inlineStr">
+    <row r="103">
+      <c r="A103" s="7" t="inlineStr">
         <is>
           <t>table:*</t>
         </is>
       </c>
-      <c r="B92" s="7" t="inlineStr">
+      <c r="B103" s="7" t="inlineStr">
         <is>
           <t>table:*  (or table:1)</t>
         </is>
       </c>
-      <c r="C92" s="7" t="inlineStr"/>
-      <c r="D92" s="7" t="inlineStr">
+      <c r="C103" s="7" t="inlineStr"/>
+      <c r="D103" s="7" t="inlineStr">
         <is>
           <t>Begin a repeating table block.</t>
         </is>
       </c>
     </row>
-    <row r="93">
-      <c r="A93" s="8" t="inlineStr">
+    <row r="104">
+      <c r="A104" s="8" t="inlineStr">
         <is>
           <t>HEADER:N</t>
         </is>
       </c>
-      <c r="B93" s="8" t="inlineStr">
+      <c r="B104" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve"> | HEADER:1 | F1 | F2</t>
         </is>
       </c>
-      <c r="C93" s="8" t="inlineStr"/>
-      <c r="D93" s="8" t="inlineStr">
+      <c r="C104" s="8" t="inlineStr"/>
+      <c r="D104" s="8" t="inlineStr">
         <is>
           <t>Strict header row template (col A must be blank).</t>
         </is>
       </c>
     </row>
-    <row r="94">
-      <c r="A94" s="8" t="inlineStr">
+    <row r="105">
+      <c r="A105" s="8" t="inlineStr">
         <is>
           <t>DATA:*</t>
         </is>
       </c>
-      <c r="B94" s="8" t="inlineStr">
+      <c r="B105" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve"> | DATA:* | F1 | F2</t>
         </is>
       </c>
-      <c r="C94" s="8" t="inlineStr"/>
-      <c r="D94" s="8" t="inlineStr">
+      <c r="C105" s="8" t="inlineStr"/>
+      <c r="D105" s="8" t="inlineStr">
         <is>
           <t>Data row template (greedy, lenient validation).</t>
         </is>
       </c>
     </row>
-    <row r="95">
-      <c r="A95" s="8" t="inlineStr">
+    <row r="106">
+      <c r="A106" s="8" t="inlineStr">
         <is>
           <t>DATA:{n,m}</t>
         </is>
       </c>
-      <c r="B95" s="8" t="inlineStr">
+      <c r="B106" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve"> | DATA:{0,15} | F1 | F2</t>
         </is>
       </c>
-      <c r="C95" s="8" t="inlineStr"/>
-      <c r="D95" s="8" t="inlineStr">
+      <c r="C106" s="8" t="inlineStr"/>
+      <c r="D106" s="8" t="inlineStr">
         <is>
           <t>Bounded data: scan at most m physical rows, warn if &lt; n.</t>
         </is>
       </c>
     </row>
-    <row r="96">
-      <c r="A96" t="inlineStr">
+    <row r="107">
+      <c r="A107" t="inlineStr">
         <is>
           <t>SKIP_IF</t>
         </is>
       </c>
-      <c r="B96" t="inlineStr">
+      <c r="B107" t="inlineStr">
         <is>
           <t xml:space="preserve"> | SKIP_IF | EMPTY | IGNORE</t>
         </is>
       </c>
-      <c r="C96" t="inlineStr"/>
-      <c r="D96" t="inlineStr">
+      <c r="C107" t="inlineStr"/>
+      <c r="D107" t="inlineStr">
         <is>
           <t>Skip row if non-IGNORE columns match. Valid with DATA:{n,m} and DATA:*.</t>
         </is>
       </c>
     </row>
-    <row r="97">
-      <c r="A97" s="8" t="inlineStr">
+    <row r="108">
+      <c r="A108" s="8" t="inlineStr">
         <is>
           <t>FOOTER:N</t>
         </is>
       </c>
-      <c r="B97" s="8" t="inlineStr">
+      <c r="B108" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve"> | FOOTER:1 | F1 | F2</t>
         </is>
       </c>
-      <c r="C97" s="8" t="inlineStr"/>
-      <c r="D97" s="8" t="inlineStr">
+      <c r="C108" s="8" t="inlineStr"/>
+      <c r="D108" s="8" t="inlineStr">
         <is>
           <t>Strict footer row template.</t>
         </is>
       </c>
     </row>
-    <row r="98">
-      <c r="A98" s="8" t="inlineStr">
+    <row r="109">
+      <c r="A109" s="8" t="inlineStr">
         <is>
           <t>SPLITTER</t>
         </is>
       </c>
-      <c r="B98" s="8" t="inlineStr">
+      <c r="B109" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve"> | SPLITTER:1</t>
         </is>
       </c>
-      <c r="C98" s="8" t="inlineStr"/>
-      <c r="D98" s="8" t="inlineStr">
+      <c r="C109" s="8" t="inlineStr"/>
+      <c r="D109" s="8" t="inlineStr">
         <is>
           <t>All columns must be blank (separator row).</t>
         </is>

</xml_diff>

<commit_message>
docs: complete TAB completion documentation across all surfaces
- CHANGELOG.md: [Unreleased] entries for TAB completion, docs rewrite,
  guide sheet redesign, and help improvements from this session.
- docs/cli-reference.md: new "Shell TAB completion" section at the top
  with bash/zsh activation instructions.
- cli.py: epilog on main parser shows activation command in --help output.
- docs_generator.py: TAB completion section added to guide sheet and
  grepxcel-guide.docx (between Available Commands and Pattern File Format).
- docs/ regenerated with the updated guide content.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K6EyxWBecbqyp9uRx7c4J8
</commit_message>
<xml_diff>
--- a/docs/pattern-reference.xlsx
+++ b/docs/pattern-reference.xlsx
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C43"/>
+  <dimension ref="A1:C47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -924,7 +924,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>REGENERATING THIS GUIDE</t>
+          <t>SHELL TAB COMPLETION</t>
         </is>
       </c>
       <c r="B40" s="3" t="n"/>
@@ -932,9 +932,9 @@
     </row>
     <row r="41">
       <c r="A41" t="inlineStr"/>
-      <c r="B41" s="5" t="inlineStr">
-        <is>
-          <t>grepxcel docs</t>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Add once to ~/.bashrc or ~/.zshrc to enable TAB completion for all commands and flags:</t>
         </is>
       </c>
     </row>
@@ -942,13 +942,38 @@
       <c r="A42" t="inlineStr"/>
       <c r="B42" s="5" t="inlineStr">
         <is>
+          <t>eval "$(register-python-argcomplete grepxcel)"</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>REGENERATING THIS GUIDE</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n"/>
+      <c r="C44" s="3" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr"/>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>grepxcel docs</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr"/>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
           <t>grepxcel docs -o /your/output/directory/</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" t="inlineStr"/>
-      <c r="B43" t="inlineStr">
+    <row r="47">
+      <c r="A47" t="inlineStr"/>
+      <c r="B47" t="inlineStr">
         <is>
           <t>Both pattern-reference.xlsx and grepxcel-guide.docx are regenerated together.</t>
         </is>

</xml_diff>

<commit_message>
chore(docs): regenerate pattern-reference.xlsx and grepxcel-guide.docx
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K6EyxWBecbqyp9uRx7c4J8
</commit_message>
<xml_diff>
--- a/docs/pattern-reference.xlsx
+++ b/docs/pattern-reference.xlsx
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C47"/>
+  <dimension ref="A1:C55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -534,7 +534,7 @@
       <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
-          <t>and grepxcel finds them reliably across any number of files.</t>
+          <t>and grepxcel attempts to extract them across any number of files.</t>
         </is>
       </c>
     </row>
@@ -546,95 +546,91 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>When data does not match the pattern, grepxcel reports it and stops — no silent errors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>QUICK START</t>
         </is>
       </c>
-      <c r="B10" s="3" t="n"/>
-      <c r="C10" s="3" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="B11" s="3" t="n"/>
+      <c r="C11" s="3" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>1  Install grepxcel</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>pip install grepxcel</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>2  Generate ready-to-run examples</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>grepxcel generate-examples -o examples/</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>3  Run your first extraction</t>
+          <t>2  Generate ready-to-run examples</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>grepxcel extract -p examples/01_simple_invoice/pattern.xlsx  examples/01_simple_invoice/data.xlsx</t>
+          <t>grepxcel generate-examples -o examples/</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>4  Write output to files</t>
+          <t>3  Run your first extraction</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>grepxcel extract -p pattern.xlsx data.xlsx -o output/</t>
+          <t>grepxcel extract -p examples/01_simple_invoice/pattern.xlsx  examples/01_simple_invoice/data.xlsx</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>4  Write output to files</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>grepxcel extract -p pattern.xlsx data.xlsx -o output/</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>5  Build your own pattern</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Use the wizard (see below) or open the pattern-reference sheet in this file</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Use the web wizard (see below) or open the pattern-reference sheet in this file</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>WIZARD — VISUAL PATTERN BUILDER</t>
         </is>
       </c>
-      <c r="B17" s="3" t="n"/>
-      <c r="C17" s="3" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Terminal wizard (keyboard)</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>grepxcel wizard data.xlsx</t>
-        </is>
-      </c>
+      <c r="B18" s="3" t="n"/>
+      <c r="C18" s="3" t="n"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -661,84 +657,79 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>grepxcel wizard data.xlsx --load-pattern pattern.xlsx</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+          <t>grepxcel web-wizard data.xlsx -p pattern.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Custom port / no auto-open</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>grepxcel web-wizard data.xlsx --port 9000 --no-browser</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>AVAILABLE COMMANDS</t>
         </is>
       </c>
-      <c r="B22" s="3" t="n"/>
-      <c r="C22" s="3" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>extract</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Extract data from Excel files using a pattern</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>grepxcel extract -p pattern.xlsx data.xlsx</t>
-        </is>
-      </c>
+      <c r="B23" s="3" t="n"/>
+      <c r="C23" s="3" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>validate-pattern</t>
+          <t>extract</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Check a pattern file without running extraction</t>
+          <t>Extract data from Excel files using a pattern</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>grepxcel validate-pattern pattern.xlsx</t>
+          <t>grepxcel extract -p pattern.xlsx data.xlsx</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>validate-pattern</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>AI-powered pattern drafter (optional)</t>
+          <t>Check a pattern file without running extraction</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>pip install 'grepxcel[suggest]'  then  grepxcel draft data.xlsx</t>
+          <t>grepxcel validate-pattern pattern.xlsx</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>wizard</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Terminal-based visual pattern builder</t>
+          <t>AI-powered pattern drafter (optional)</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>grepxcel wizard data.xlsx</t>
+          <t>pip install 'grepxcel[suggest]'  then  grepxcel draft data.xlsx</t>
         </is>
       </c>
     </row>
@@ -762,220 +753,304 @@
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>docs</t>
+          <t>test</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Regenerate this guide + grepxcel-guide.docx</t>
+          <t>Run pattern against a folder — pass/warn/fail report</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>grepxcel docs -o /output/directory/</t>
+          <t>grepxcel test -p pattern.xlsx samples/</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>generate-examples</t>
+          <t>lint</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Write 4 ready-to-run example files to a directory</t>
+          <t>Inspect an Excel file before writing a pattern</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>grepxcel generate-examples -o examples/</t>
+          <t>grepxcel lint data.xlsx</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>lint</t>
+          <t>schema</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Inspect an Excel file before writing a pattern</t>
+          <t>Generate JSON Schema from a pattern file</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>grepxcel lint data.xlsx</t>
+          <t>grepxcel schema pattern.xlsx</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>schema</t>
+          <t>docs</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Generate JSON Schema from a pattern file</t>
+          <t>Regenerate this guide + grepxcel-guide.docx</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>grepxcel schema pattern.xlsx</t>
+          <t>grepxcel docs -o /output/directory/</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>generate-examples</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Write 4 ready-to-run example files to a directory</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>grepxcel generate-examples -o examples/</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>doctor</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Check your environment is ready</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>grepxcel doctor</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>quickstart</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Guided tutorial in your terminal</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>grepxcel quickstart</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>PATTERN FILE COLOUR KEY</t>
         </is>
       </c>
-      <c r="B33" s="3" t="n"/>
-      <c r="C33" s="3" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="6" t="inlineStr">
-        <is>
-          <t>doc:</t>
-        </is>
-      </c>
-      <c r="B34" s="6" t="inlineStr">
+      <c r="B36" s="3" t="n"/>
+      <c r="C36" s="3" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
         <is>
           <t>yellow</t>
         </is>
       </c>
-      <c r="C34" s="6" t="inlineStr">
+      <c r="C37" s="6" t="inlineStr">
         <is>
           <t>Comment rows — ignored by the engine</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="7" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="7" t="inlineStr">
         <is>
           <t>lbl:</t>
         </is>
       </c>
-      <c r="B35" s="7" t="inlineStr">
+      <c r="B38" s="7" t="inlineStr">
         <is>
           <t>blue</t>
         </is>
       </c>
-      <c r="C35" s="7" t="inlineStr">
+      <c r="C38" s="7" t="inlineStr">
         <is>
           <t>Anchor labels — matched for position, never extracted</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="8" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="8" t="inlineStr">
         <is>
           <t>var:</t>
         </is>
       </c>
-      <c r="B36" s="8" t="inlineStr">
+      <c r="B39" s="8" t="inlineStr">
         <is>
           <t>green</t>
         </is>
       </c>
-      <c r="C36" s="8" t="inlineStr">
+      <c r="C39" s="8" t="inlineStr">
         <is>
           <t>Variables — extracted and written to output JSON</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="9" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="9" t="inlineStr">
         <is>
           <t>config:</t>
         </is>
       </c>
-      <c r="B37" s="9" t="inlineStr">
+      <c r="B40" s="9" t="inlineStr">
         <is>
           <t>orange</t>
         </is>
       </c>
-      <c r="C37" s="9" t="inlineStr">
+      <c r="C40" s="9" t="inlineStr">
         <is>
           <t>Global settings (read.direction, currency.sign, ...)</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="10" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="10" t="inlineStr">
         <is>
           <t>cell: / table:</t>
         </is>
       </c>
-      <c r="B38" s="10" t="inlineStr">
+      <c r="B41" s="10" t="inlineStr">
         <is>
           <t>lavender</t>
         </is>
       </c>
-      <c r="C38" s="10" t="inlineStr">
+      <c r="C41" s="10" t="inlineStr">
         <is>
           <t>Instructions — cursor movement and table scanning</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
         <is>
           <t>SHELL TAB COMPLETION</t>
         </is>
       </c>
-      <c r="B40" s="3" t="n"/>
-      <c r="C40" s="3" t="n"/>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr"/>
-      <c r="B41" t="inlineStr">
+      <c r="B43" s="3" t="n"/>
+      <c r="C43" s="3" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr"/>
+      <c r="B44" t="inlineStr">
         <is>
           <t>Add once to ~/.bashrc or ~/.zshrc to enable TAB completion for all commands and flags:</t>
         </is>
       </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr"/>
-      <c r="B42" s="5" t="inlineStr">
-        <is>
-          <t>eval "$(register-python-argcomplete grepxcel)"</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>REGENERATING THIS GUIDE</t>
-        </is>
-      </c>
-      <c r="B44" s="3" t="n"/>
-      <c r="C44" s="3" t="n"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr"/>
       <c r="B45" s="5" t="inlineStr">
         <is>
+          <t>eval "$(register-python-argcomplete grepxcel)"</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>REGENERATING THIS GUIDE</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n"/>
+      <c r="C47" s="3" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr"/>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
           <t>grepxcel docs</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" t="inlineStr"/>
-      <c r="B46" s="5" t="inlineStr">
+    <row r="49">
+      <c r="A49" t="inlineStr"/>
+      <c r="B49" s="5" t="inlineStr">
         <is>
           <t>grepxcel docs -o /your/output/directory/</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" t="inlineStr"/>
-      <c r="B47" t="inlineStr">
+    <row r="50">
+      <c r="A50" t="inlineStr"/>
+      <c r="B50" t="inlineStr">
         <is>
           <t>Both pattern-reference.xlsx and grepxcel-guide.docx are regenerated together.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>GENERATED BY</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n"/>
+      <c r="C52" s="3" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr"/>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>grepxcel 0.4.0rc1</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr"/>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Generated:  2026-09-20 11:22 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr"/>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Executable: /home/scpg-dev/dev/projects/grepxcel/.venv/bin/grepxcel</t>
         </is>
       </c>
     </row>
@@ -990,7 +1065,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F118"/>
+  <dimension ref="A1:F123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3003,6 +3078,62 @@
         </is>
       </c>
     </row>
+    <row r="120">
+      <c r="A120" s="6" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B120" s="6" t="inlineStr"/>
+      <c r="C120" s="6" t="inlineStr"/>
+      <c r="D120" s="6" t="inlineStr">
+        <is>
+          <t>── GENERATED BY ──────────────────────────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="6" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B121" s="6" t="inlineStr"/>
+      <c r="C121" s="6" t="inlineStr"/>
+      <c r="D121" s="6" t="inlineStr">
+        <is>
+          <t>grepxcel 0.4.0rc1</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="6" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B122" s="6" t="inlineStr"/>
+      <c r="C122" s="6" t="inlineStr"/>
+      <c r="D122" s="6" t="inlineStr">
+        <is>
+          <t>Generated:  2026-09-20 11:22 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="6" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B123" s="6" t="inlineStr"/>
+      <c r="C123" s="6" t="inlineStr"/>
+      <c r="D123" s="6" t="inlineStr">
+        <is>
+          <t>Executable: /home/scpg-dev/dev/projects/grepxcel/.venv/bin/grepxcel</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: document table:{n,m} in the generated pattern reference
The generated pattern-reference.xlsx / grepxcel-guide.docx described
DATA:{n,m} but had no entry for the new table:N / table:{n,m} multiplicity
semantics. Adds a doc line and a quick-reference row, and fixes the
fill-colour key derivation (rstrip(':*1') never stripped the trailing '}'
so a bracketed table row would have rendered unstyled). Artifacts
regenerated with `grepxcel docs -o docs/ --force` so CI's byte-diff check
stays current.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K6EyxWBecbqyp9uRx7c4J8
</commit_message>
<xml_diff>
--- a/docs/pattern-reference.xlsx
+++ b/docs/pattern-reference.xlsx
@@ -1034,7 +1034,7 @@
       <c r="A53" t="inlineStr"/>
       <c r="B53" t="inlineStr">
         <is>
-          <t>grepxcel 0.4.0rc1</t>
+          <t>grepxcel 0.4.2rc2</t>
         </is>
       </c>
     </row>
@@ -1042,7 +1042,7 @@
       <c r="A54" t="inlineStr"/>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Generated:  2026-09-20 11:22 UTC</t>
+          <t>Generated:  2026-09-26 18:27 UTC</t>
         </is>
       </c>
     </row>
@@ -1065,7 +1065,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F123"/>
+  <dimension ref="A1:F125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2477,42 +2477,29 @@
       <c r="D81" s="6" t="inlineStr"/>
       <c r="E81" s="6" t="inlineStr">
         <is>
-          <t>Use table:1 when exactly one instance is expected.</t>
+          <t>table:1 stops after exactly one instance; table:N after exactly N (warns if fewer are found).</t>
         </is>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="10" t="inlineStr">
+      <c r="A82" s="6" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B82" s="6" t="inlineStr"/>
+      <c r="C82" s="6" t="inlineStr"/>
+      <c r="D82" s="6" t="inlineStr"/>
+      <c r="E82" s="6" t="inlineStr">
+        <is>
+          <t>table:{n,m} scans at most m instances; warns if fewer than n are found — same bounds as DATA:{n,m}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="10" t="inlineStr">
         <is>
           <t>table:*</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" s="12" t="n"/>
-      <c r="B83" s="12" t="inlineStr">
-        <is>
-          <t>HEADER:1</t>
-        </is>
-      </c>
-      <c r="C83" s="12" t="inlineStr">
-        <is>
-          <t>col_item</t>
-        </is>
-      </c>
-      <c r="D83" s="12" t="inlineStr">
-        <is>
-          <t>col_qty</t>
-        </is>
-      </c>
-      <c r="E83" s="12" t="inlineStr">
-        <is>
-          <t>col_price</t>
-        </is>
-      </c>
-      <c r="F83" s="12" t="inlineStr">
-        <is>
-          <t>col_total</t>
         </is>
       </c>
     </row>
@@ -2520,27 +2507,27 @@
       <c r="A84" s="12" t="n"/>
       <c r="B84" s="12" t="inlineStr">
         <is>
-          <t>DATA:*</t>
+          <t>HEADER:1</t>
         </is>
       </c>
       <c r="C84" s="12" t="inlineStr">
         <is>
-          <t>line.item</t>
+          <t>col_item</t>
         </is>
       </c>
       <c r="D84" s="12" t="inlineStr">
         <is>
-          <t>line.qty</t>
+          <t>col_qty</t>
         </is>
       </c>
       <c r="E84" s="12" t="inlineStr">
         <is>
-          <t>line.price</t>
+          <t>col_price</t>
         </is>
       </c>
       <c r="F84" s="12" t="inlineStr">
         <is>
-          <t>line.total</t>
+          <t>col_total</t>
         </is>
       </c>
     </row>
@@ -2548,42 +2535,55 @@
       <c r="A85" s="12" t="n"/>
       <c r="B85" s="12" t="inlineStr">
         <is>
+          <t>DATA:*</t>
+        </is>
+      </c>
+      <c r="C85" s="12" t="inlineStr">
+        <is>
+          <t>line.item</t>
+        </is>
+      </c>
+      <c r="D85" s="12" t="inlineStr">
+        <is>
+          <t>line.qty</t>
+        </is>
+      </c>
+      <c r="E85" s="12" t="inlineStr">
+        <is>
+          <t>line.price</t>
+        </is>
+      </c>
+      <c r="F85" s="12" t="inlineStr">
+        <is>
+          <t>line.total</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="12" t="n"/>
+      <c r="B86" s="12" t="inlineStr">
+        <is>
           <t>FOOTER:1</t>
         </is>
       </c>
-      <c r="C85" s="12" t="inlineStr">
+      <c r="C86" s="12" t="inlineStr">
         <is>
           <t>footer.label</t>
         </is>
       </c>
-      <c r="D85" s="12" t="inlineStr">
+      <c r="D86" s="12" t="inlineStr">
         <is>
           <t>IGNORE</t>
         </is>
       </c>
-      <c r="E85" s="12" t="inlineStr">
+      <c r="E86" s="12" t="inlineStr">
         <is>
           <t>IGNORE</t>
         </is>
       </c>
-      <c r="F85" s="12" t="inlineStr">
+      <c r="F86" s="12" t="inlineStr">
         <is>
           <t>footer.value</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" s="6" t="inlineStr">
-        <is>
-          <t>doc:</t>
-        </is>
-      </c>
-      <c r="B86" s="6" t="inlineStr"/>
-      <c r="C86" s="6" t="inlineStr"/>
-      <c r="D86" s="6" t="inlineStr"/>
-      <c r="E86" s="6" t="inlineStr">
-        <is>
-          <t>HEADER/FOOTER are strict: wrong or missing value = no match.</t>
         </is>
       </c>
     </row>
@@ -2598,7 +2598,7 @@
       <c r="D87" s="6" t="inlineStr"/>
       <c r="E87" s="6" t="inlineStr">
         <is>
-          <t>DATA rows are lenient: wrong value emits a warning but extraction continues.</t>
+          <t>HEADER/FOOTER are strict: wrong or missing value = no match.</t>
         </is>
       </c>
     </row>
@@ -2613,7 +2613,7 @@
       <c r="D88" s="6" t="inlineStr"/>
       <c r="E88" s="6" t="inlineStr">
         <is>
-          <t>EMPTY column keyword: cell must be blank. IGNORE: consume without matching.</t>
+          <t>DATA rows are lenient: wrong value emits a warning but extraction continues.</t>
         </is>
       </c>
     </row>
@@ -2628,7 +2628,7 @@
       <c r="D89" s="6" t="inlineStr"/>
       <c r="E89" s="6" t="inlineStr">
         <is>
-          <t>── BOUNDED DATA + SKIP_IF (fixed-slot templates) ───────────────────────</t>
+          <t>EMPTY column keyword: cell must be blank. IGNORE: consume without matching.</t>
         </is>
       </c>
     </row>
@@ -2643,7 +2643,7 @@
       <c r="D90" s="6" t="inlineStr"/>
       <c r="E90" s="6" t="inlineStr">
         <is>
-          <t>Use DATA:{n,m} when the template pre-allocates a fixed number of rows.</t>
+          <t>── BOUNDED DATA + SKIP_IF (fixed-slot templates) ───────────────────────</t>
         </is>
       </c>
     </row>
@@ -2658,7 +2658,7 @@
       <c r="D91" s="6" t="inlineStr"/>
       <c r="E91" s="6" t="inlineStr">
         <is>
-          <t>n = min total physical rows expected, m = max total rows to scan.</t>
+          <t>Use DATA:{n,m} when the template pre-allocates a fixed number of rows.</t>
         </is>
       </c>
     </row>
@@ -2673,7 +2673,7 @@
       <c r="D92" s="6" t="inlineStr"/>
       <c r="E92" s="6" t="inlineStr">
         <is>
-          <t>SKIP_IF: rows matching the condition are silently excluded from output</t>
+          <t>n = min total physical rows expected, m = max total rows to scan.</t>
         </is>
       </c>
     </row>
@@ -2688,7 +2688,7 @@
       <c r="D93" s="6" t="inlineStr"/>
       <c r="E93" s="6" t="inlineStr">
         <is>
-          <t>but still count toward the {n,m} bounds.</t>
+          <t>SKIP_IF: rows matching the condition are silently excluded from output</t>
         </is>
       </c>
     </row>
@@ -2703,32 +2703,29 @@
       <c r="D94" s="6" t="inlineStr"/>
       <c r="E94" s="6" t="inlineStr">
         <is>
+          <t>but still count toward the {n,m} bounds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="6" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B95" s="6" t="inlineStr"/>
+      <c r="C95" s="6" t="inlineStr"/>
+      <c r="D95" s="6" t="inlineStr"/>
+      <c r="E95" s="6" t="inlineStr">
+        <is>
           <t>SKIP_IF is valid with DATA:{n,m} (rows count toward bounds) and DATA:* (rows filtered, scan continues).</t>
         </is>
       </c>
     </row>
-    <row r="95">
-      <c r="A95" s="10" t="inlineStr">
+    <row r="96">
+      <c r="A96" s="10" t="inlineStr">
         <is>
           <t>table:1</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" s="12" t="n"/>
-      <c r="B96" s="12" t="inlineStr">
-        <is>
-          <t>HEADER:1</t>
-        </is>
-      </c>
-      <c r="C96" s="12" t="inlineStr">
-        <is>
-          <t>col_item</t>
-        </is>
-      </c>
-      <c r="D96" s="12" t="inlineStr">
-        <is>
-          <t>col_qty</t>
         </is>
       </c>
     </row>
@@ -2736,17 +2733,17 @@
       <c r="A97" s="12" t="n"/>
       <c r="B97" s="12" t="inlineStr">
         <is>
-          <t>SKIP_IF</t>
+          <t>HEADER:1</t>
         </is>
       </c>
       <c r="C97" s="12" t="inlineStr">
         <is>
-          <t>EMPTY</t>
+          <t>col_item</t>
         </is>
       </c>
       <c r="D97" s="12" t="inlineStr">
         <is>
-          <t>IGNORE</t>
+          <t>col_qty</t>
         </is>
       </c>
     </row>
@@ -2754,17 +2751,17 @@
       <c r="A98" s="12" t="n"/>
       <c r="B98" s="12" t="inlineStr">
         <is>
-          <t>DATA:{0,15}</t>
+          <t>SKIP_IF</t>
         </is>
       </c>
       <c r="C98" s="12" t="inlineStr">
         <is>
-          <t>line.item</t>
+          <t>EMPTY</t>
         </is>
       </c>
       <c r="D98" s="12" t="inlineStr">
         <is>
-          <t>line.qty</t>
+          <t>IGNORE</t>
         </is>
       </c>
     </row>
@@ -2772,39 +2769,42 @@
       <c r="A99" s="12" t="n"/>
       <c r="B99" s="12" t="inlineStr">
         <is>
+          <t>DATA:{0,15}</t>
+        </is>
+      </c>
+      <c r="C99" s="12" t="inlineStr">
+        <is>
+          <t>line.item</t>
+        </is>
+      </c>
+      <c r="D99" s="12" t="inlineStr">
+        <is>
+          <t>line.qty</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="12" t="n"/>
+      <c r="B100" s="12" t="inlineStr">
+        <is>
           <t>FOOTER:1</t>
         </is>
       </c>
-      <c r="C99" s="12" t="inlineStr">
+      <c r="C100" s="12" t="inlineStr">
         <is>
           <t>lbl_total</t>
         </is>
       </c>
-      <c r="D99" s="12" t="inlineStr">
+      <c r="D100" s="12" t="inlineStr">
         <is>
           <t>inv.total</t>
         </is>
       </c>
     </row>
-    <row r="101">
-      <c r="A101" s="11" t="inlineStr">
+    <row r="102">
+      <c r="A102" s="11" t="inlineStr">
         <is>
           <t>END:</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" s="6" t="inlineStr">
-        <is>
-          <t>doc:</t>
-        </is>
-      </c>
-      <c r="B103" s="6" t="inlineStr"/>
-      <c r="C103" s="6" t="inlineStr"/>
-      <c r="D103" s="6" t="inlineStr"/>
-      <c r="E103" s="6" t="inlineStr">
-        <is>
-          <t>── QUICK REFERENCE ──────────────────────────────────────────────</t>
         </is>
       </c>
     </row>
@@ -2814,87 +2814,84 @@
           <t>doc:</t>
         </is>
       </c>
-      <c r="B104" s="6" t="inlineStr">
+      <c r="B104" s="6" t="inlineStr"/>
+      <c r="C104" s="6" t="inlineStr"/>
+      <c r="D104" s="6" t="inlineStr"/>
+      <c r="E104" s="6" t="inlineStr">
+        <is>
+          <t>── QUICK REFERENCE ──────────────────────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="6" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B105" s="6" t="inlineStr">
         <is>
           <t>doc: | free text</t>
         </is>
       </c>
-      <c r="C104" s="6" t="inlineStr"/>
-      <c r="D104" s="6" t="inlineStr">
+      <c r="C105" s="6" t="inlineStr"/>
+      <c r="D105" s="6" t="inlineStr">
         <is>
           <t>Inline comment. Ignored by engine.</t>
         </is>
       </c>
     </row>
-    <row r="105">
-      <c r="A105" s="9" t="inlineStr">
+    <row r="106">
+      <c r="A106" s="9" t="inlineStr">
         <is>
           <t>config:</t>
         </is>
       </c>
-      <c r="B105" s="9" t="inlineStr">
+      <c r="B106" s="9" t="inlineStr">
         <is>
           <t>config: | key | value</t>
         </is>
       </c>
-      <c r="C105" s="9" t="inlineStr"/>
-      <c r="D105" s="9" t="inlineStr">
+      <c r="C106" s="9" t="inlineStr"/>
+      <c r="D106" s="9" t="inlineStr">
         <is>
           <t>Global setting. Keys: read.direction, currency.sign, empty.aliases, ignore.case</t>
         </is>
       </c>
     </row>
-    <row r="106">
-      <c r="A106" s="7" t="inlineStr">
+    <row r="107">
+      <c r="A107" s="7" t="inlineStr">
         <is>
           <t>lbl:</t>
         </is>
       </c>
-      <c r="B106" s="7" t="inlineStr">
+      <c r="B107" s="7" t="inlineStr">
         <is>
           <t>lbl: | name | type | regex</t>
         </is>
       </c>
-      <c r="C106" s="7" t="inlineStr"/>
-      <c r="D106" s="7" t="inlineStr">
+      <c r="C107" s="7" t="inlineStr"/>
+      <c r="D107" s="7" t="inlineStr">
         <is>
           <t>Anchor label. Matched but never in output.</t>
         </is>
       </c>
     </row>
-    <row r="107">
-      <c r="A107" s="8" t="inlineStr">
+    <row r="108">
+      <c r="A108" s="8" t="inlineStr">
         <is>
           <t>var:</t>
         </is>
       </c>
-      <c r="B107" s="8" t="inlineStr">
+      <c r="B108" s="8" t="inlineStr">
         <is>
           <t>var: | name | type | regex</t>
         </is>
       </c>
-      <c r="C107" s="8" t="inlineStr"/>
-      <c r="D107" s="8" t="inlineStr">
+      <c r="C108" s="8" t="inlineStr"/>
+      <c r="D108" s="8" t="inlineStr">
         <is>
           <t>Extracted variable. Use dot notation for nesting.</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" t="inlineStr">
-        <is>
-          <t>cell:next</t>
-        </is>
-      </c>
-      <c r="B108" t="inlineStr">
-        <is>
-          <t>cell:next | FieldName</t>
-        </is>
-      </c>
-      <c r="C108" t="inlineStr"/>
-      <c r="D108" t="inlineStr">
-        <is>
-          <t>Read next non-empty cell (alias: cell:1).</t>
         </is>
       </c>
     </row>
@@ -2906,13 +2903,13 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>cell:next | IGNORE</t>
+          <t>cell:next | FieldName</t>
         </is>
       </c>
       <c r="C109" t="inlineStr"/>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Skip next non-empty cell without capturing.</t>
+          <t>Read next non-empty cell (alias: cell:1).</t>
         </is>
       </c>
     </row>
@@ -2924,185 +2921,193 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>cell:B5 | FieldName</t>
+          <t>cell:next | IGNORE</t>
         </is>
       </c>
       <c r="C110" t="inlineStr"/>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Jump directly to B5 (absolute reference). Ordering must be forward.</t>
+          <t>Skip next non-empty cell without capturing.</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>seek:</t>
+          <t>cell:next</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>seek:G5</t>
+          <t>cell:B5 | FieldName</t>
         </is>
       </c>
       <c r="C111" t="inlineStr"/>
       <c r="D111" t="inlineStr">
         <is>
+          <t>Jump directly to B5 (absolute reference). Ordering must be forward.</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>seek:</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>seek:G5</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr"/>
+      <c r="D112" t="inlineStr">
+        <is>
           <t>Reposition cursor to G5 without reading it. Resets abs-ref ordering constraint.</t>
         </is>
       </c>
     </row>
-    <row r="112">
-      <c r="A112" s="10" t="inlineStr">
+    <row r="113">
+      <c r="A113" s="10" t="inlineStr">
         <is>
           <t>table:*</t>
         </is>
       </c>
-      <c r="B112" s="10" t="inlineStr">
-        <is>
-          <t>table:*  (or table:1)</t>
-        </is>
-      </c>
-      <c r="C112" s="10" t="inlineStr"/>
-      <c r="D112" s="10" t="inlineStr">
+      <c r="B113" s="10" t="inlineStr">
+        <is>
+          <t>table:*  (or table:1, table:N)</t>
+        </is>
+      </c>
+      <c r="C113" s="10" t="inlineStr"/>
+      <c r="D113" s="10" t="inlineStr">
         <is>
           <t>Begin a repeating table block.</t>
         </is>
       </c>
     </row>
-    <row r="113">
-      <c r="A113" s="12" t="inlineStr">
-        <is>
-          <t>HEADER:N</t>
-        </is>
-      </c>
-      <c r="B113" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> | HEADER:1 | F1 | F2</t>
-        </is>
-      </c>
-      <c r="C113" s="12" t="inlineStr"/>
-      <c r="D113" s="12" t="inlineStr">
-        <is>
-          <t>Strict header row template (col A must be blank).</t>
-        </is>
-      </c>
-    </row>
     <row r="114">
-      <c r="A114" s="12" t="inlineStr">
-        <is>
-          <t>DATA:*</t>
-        </is>
-      </c>
-      <c r="B114" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> | DATA:* | F1 | F2</t>
-        </is>
-      </c>
-      <c r="C114" s="12" t="inlineStr"/>
-      <c r="D114" s="12" t="inlineStr">
-        <is>
-          <t>Data row template (greedy, lenient validation).</t>
+      <c r="A114" s="10" t="inlineStr">
+        <is>
+          <t>table:{n,m}</t>
+        </is>
+      </c>
+      <c r="B114" s="10" t="inlineStr">
+        <is>
+          <t>table:{2,5}</t>
+        </is>
+      </c>
+      <c r="C114" s="10" t="inlineStr"/>
+      <c r="D114" s="10" t="inlineStr">
+        <is>
+          <t>Bounded table: scan at most m instances, warn if &lt; n.</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="12" t="inlineStr">
         <is>
-          <t>DATA:{n,m}</t>
+          <t>HEADER:N</t>
         </is>
       </c>
       <c r="B115" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | DATA:{0,15} | F1 | F2</t>
+          <t xml:space="preserve"> | HEADER:1 | F1 | F2</t>
         </is>
       </c>
       <c r="C115" s="12" t="inlineStr"/>
       <c r="D115" s="12" t="inlineStr">
         <is>
-          <t>Bounded data: scan at most m physical rows, warn if &lt; n.</t>
+          <t>Strict header row template (col A must be blank).</t>
         </is>
       </c>
     </row>
     <row r="116">
-      <c r="A116" t="inlineStr">
-        <is>
-          <t>SKIP_IF</t>
-        </is>
-      </c>
-      <c r="B116" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> | SKIP_IF | EMPTY | IGNORE</t>
-        </is>
-      </c>
-      <c r="C116" t="inlineStr"/>
-      <c r="D116" t="inlineStr">
-        <is>
-          <t>Skip row if non-IGNORE columns match. Valid with DATA:{n,m} and DATA:*.</t>
+      <c r="A116" s="12" t="inlineStr">
+        <is>
+          <t>DATA:*</t>
+        </is>
+      </c>
+      <c r="B116" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> | DATA:* | F1 | F2</t>
+        </is>
+      </c>
+      <c r="C116" s="12" t="inlineStr"/>
+      <c r="D116" s="12" t="inlineStr">
+        <is>
+          <t>Data row template (greedy, lenient validation).</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="12" t="inlineStr">
         <is>
-          <t>FOOTER:N</t>
+          <t>DATA:{n,m}</t>
         </is>
       </c>
       <c r="B117" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | FOOTER:1 | F1 | F2</t>
+          <t xml:space="preserve"> | DATA:{0,15} | F1 | F2</t>
         </is>
       </c>
       <c r="C117" s="12" t="inlineStr"/>
       <c r="D117" s="12" t="inlineStr">
         <is>
+          <t>Bounded data: scan at most m physical rows, warn if &lt; n.</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>SKIP_IF</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> | SKIP_IF | EMPTY | IGNORE</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr"/>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Skip row if non-IGNORE columns match. Valid with DATA:{n,m} and DATA:*.</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="12" t="inlineStr">
+        <is>
+          <t>FOOTER:N</t>
+        </is>
+      </c>
+      <c r="B119" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> | FOOTER:1 | F1 | F2</t>
+        </is>
+      </c>
+      <c r="C119" s="12" t="inlineStr"/>
+      <c r="D119" s="12" t="inlineStr">
+        <is>
           <t>Strict footer row template.</t>
         </is>
       </c>
     </row>
-    <row r="118">
-      <c r="A118" s="12" t="inlineStr">
+    <row r="120">
+      <c r="A120" s="12" t="inlineStr">
         <is>
           <t>SPLITTER</t>
         </is>
       </c>
-      <c r="B118" s="12" t="inlineStr">
+      <c r="B120" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve"> | SPLITTER:1</t>
         </is>
       </c>
-      <c r="C118" s="12" t="inlineStr"/>
-      <c r="D118" s="12" t="inlineStr">
+      <c r="C120" s="12" t="inlineStr"/>
+      <c r="D120" s="12" t="inlineStr">
         <is>
           <t>All columns must be blank (separator row).</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" s="6" t="inlineStr">
-        <is>
-          <t>doc:</t>
-        </is>
-      </c>
-      <c r="B120" s="6" t="inlineStr"/>
-      <c r="C120" s="6" t="inlineStr"/>
-      <c r="D120" s="6" t="inlineStr">
-        <is>
-          <t>── GENERATED BY ──────────────────────────────────────────────────</t>
-        </is>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" s="6" t="inlineStr">
-        <is>
-          <t>doc:</t>
-        </is>
-      </c>
-      <c r="B121" s="6" t="inlineStr"/>
-      <c r="C121" s="6" t="inlineStr"/>
-      <c r="D121" s="6" t="inlineStr">
-        <is>
-          <t>grepxcel 0.4.0rc1</t>
         </is>
       </c>
     </row>
@@ -3116,7 +3121,7 @@
       <c r="C122" s="6" t="inlineStr"/>
       <c r="D122" s="6" t="inlineStr">
         <is>
-          <t>Generated:  2026-09-20 11:22 UTC</t>
+          <t>── GENERATED BY ──────────────────────────────────────────────────</t>
         </is>
       </c>
     </row>
@@ -3129,6 +3134,34 @@
       <c r="B123" s="6" t="inlineStr"/>
       <c r="C123" s="6" t="inlineStr"/>
       <c r="D123" s="6" t="inlineStr">
+        <is>
+          <t>grepxcel 0.4.2rc2</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="6" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B124" s="6" t="inlineStr"/>
+      <c r="C124" s="6" t="inlineStr"/>
+      <c r="D124" s="6" t="inlineStr">
+        <is>
+          <t>Generated:  2026-09-26 18:27 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="6" t="inlineStr">
+        <is>
+          <t>doc:</t>
+        </is>
+      </c>
+      <c r="B125" s="6" t="inlineStr"/>
+      <c r="C125" s="6" t="inlineStr"/>
+      <c r="D125" s="6" t="inlineStr">
         <is>
           <t>Executable: /home/scpg-dev/dev/projects/grepxcel/.venv/bin/grepxcel</t>
         </is>

</xml_diff>